<commit_message>
Improved code for summarising nutrients, fit to multivariate linear model
</commit_message>
<xml_diff>
--- a/data_cache/streams_2019lulc.xlsx
+++ b/data_cache/streams_2019lulc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/530e20b7f6c3b906/Documents/KC-Streams-Analysis/data_cache/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{E3052FD2-981D-4E2C-8B81-FC6F18F19128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DF5573F-EEEC-47D5-8EA4-6B1422A8E3FC}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="8_{E3052FD2-981D-4E2C-8B81-FC6F18F19128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F914C5F-E4F1-4D1A-9BCF-EF12C52A3862}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14856" activeTab="1" xr2:uid="{B79C8CA6-09B2-4EB5-862A-BB01EB8BD711}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="182">
   <si>
     <t>Open Water</t>
   </si>
@@ -580,6 +580,9 @@
   </si>
   <si>
     <t>Wetlands, Total</t>
+  </si>
+  <si>
+    <t>Agriculture, Total</t>
   </si>
 </sst>
 </file>
@@ -685,6 +688,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7087,7 +7094,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DA31AB4-F286-4205-A346-ED4D5FE79DEC}">
-  <dimension ref="A1:U99"/>
+  <dimension ref="A1:V99"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
@@ -7106,14 +7113,15 @@
     <col min="14" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.109375" customWidth="1"/>
-    <col min="20" max="20" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.109375" customWidth="1"/>
+    <col min="18" max="18" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.109375" customWidth="1"/>
+    <col min="21" max="21" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>15</v>
       </c>
@@ -7163,22 +7171,25 @@
         <v>11</v>
       </c>
       <c r="Q1" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="R1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="T1" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="U1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="V1" s="4" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -7230,23 +7241,27 @@
         <v>1.1662054947120657</v>
       </c>
       <c r="Q2" s="5">
+        <f>SUM(R2:S2)</f>
+        <v>4.4267387572421546</v>
+      </c>
+      <c r="R2" s="5">
         <v>4.350742300330098</v>
       </c>
-      <c r="R2" s="5">
+      <c r="S2" s="5">
         <v>7.5996456912056962E-2</v>
       </c>
-      <c r="S2" s="5">
-        <f>SUM(T2:U2)</f>
+      <c r="T2" s="5">
+        <f>SUM(U2:V2)</f>
         <v>2.2674592533914972</v>
       </c>
-      <c r="T2" s="5">
+      <c r="U2" s="5">
         <v>1.7244393341276754</v>
       </c>
-      <c r="U2" s="5">
+      <c r="V2" s="5">
         <v>0.54301991926382176</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -7298,23 +7313,27 @@
         <v>1.1853685102172939</v>
       </c>
       <c r="Q3" s="5">
+        <f t="shared" ref="Q3:Q66" si="2">SUM(R3:S3)</f>
+        <v>4.5057562376935421</v>
+      </c>
+      <c r="R3" s="5">
         <v>4.4283508023270803</v>
       </c>
-      <c r="R3" s="5">
+      <c r="S3" s="5">
         <v>7.7405435366461467E-2</v>
       </c>
-      <c r="S3" s="5">
-        <f t="shared" ref="S3:S66" si="2">SUM(T3:U3)</f>
+      <c r="T3" s="5">
+        <f t="shared" ref="T3:T66" si="3">SUM(U3:V3)</f>
         <v>2.2963860825176208</v>
       </c>
-      <c r="T3" s="5">
+      <c r="U3" s="5">
         <v>1.7482155402400237</v>
       </c>
-      <c r="U3" s="5">
+      <c r="V3" s="5">
         <v>0.54817054227759721</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -7366,23 +7385,27 @@
         <v>1.1947770573356262</v>
       </c>
       <c r="Q4" s="5">
+        <f t="shared" si="2"/>
+        <v>4.5435183870509723</v>
+      </c>
+      <c r="R4" s="5">
         <v>4.4654642269295115</v>
       </c>
-      <c r="R4" s="5">
+      <c r="S4" s="5">
         <v>7.8054160121460978E-2</v>
       </c>
-      <c r="S4" s="5">
-        <f t="shared" si="2"/>
+      <c r="T4" s="5">
+        <f t="shared" si="3"/>
         <v>2.3122511976693434</v>
       </c>
-      <c r="T4" s="5">
+      <c r="U4" s="5">
         <v>1.762416358469177</v>
       </c>
-      <c r="U4" s="5">
+      <c r="V4" s="5">
         <v>0.54983483920016651</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -7434,23 +7457,27 @@
         <v>1.2011038763344235</v>
       </c>
       <c r="Q5" s="5">
+        <f t="shared" si="2"/>
+        <v>4.5679569146762216</v>
+      </c>
+      <c r="R5" s="5">
         <v>4.4894647499167109</v>
       </c>
-      <c r="R5" s="5">
+      <c r="S5" s="5">
         <v>7.8492164759511041E-2</v>
       </c>
-      <c r="S5" s="5">
-        <f t="shared" si="2"/>
+      <c r="T5" s="5">
+        <f t="shared" si="3"/>
         <v>2.3228845832776184</v>
       </c>
-      <c r="T5" s="5">
+      <c r="U5" s="5">
         <v>1.7722306959512699</v>
       </c>
-      <c r="U5" s="5">
+      <c r="V5" s="5">
         <v>0.55065388732634835</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -7502,23 +7529,27 @@
         <v>1.2750369945094489</v>
       </c>
       <c r="Q6" s="5">
+        <f t="shared" si="2"/>
+        <v>4.8202026409632328</v>
+      </c>
+      <c r="R6" s="5">
         <v>4.7389360136495595</v>
       </c>
-      <c r="R6" s="5">
+      <c r="S6" s="5">
         <v>8.1266627313673012E-2</v>
       </c>
-      <c r="S6" s="5">
-        <f t="shared" si="2"/>
+      <c r="T6" s="5">
+        <f t="shared" si="3"/>
         <v>2.3196972514898881</v>
       </c>
-      <c r="T6" s="5">
+      <c r="U6" s="5">
         <v>1.8101029377279305</v>
       </c>
-      <c r="U6" s="5">
+      <c r="V6" s="5">
         <v>0.50959431376195752</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -7570,23 +7601,27 @@
         <v>7.3952858986059092E-2</v>
       </c>
       <c r="Q7" s="5">
+        <f t="shared" si="2"/>
+        <v>1.2210089058123801</v>
+      </c>
+      <c r="R7" s="5">
         <v>1.1675110929288479</v>
       </c>
-      <c r="R7" s="5">
+      <c r="S7" s="5">
         <v>5.3497812883532121E-2</v>
       </c>
-      <c r="S7" s="5">
-        <f t="shared" si="2"/>
+      <c r="T7" s="5">
+        <f t="shared" si="3"/>
         <v>2.71422727129685</v>
       </c>
-      <c r="T7" s="5">
+      <c r="U7" s="5">
         <v>1.2493312773389558</v>
       </c>
-      <c r="U7" s="5">
+      <c r="V7" s="5">
         <v>1.464895993957894</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -7638,23 +7673,27 @@
         <v>2.6204494568372172</v>
       </c>
       <c r="Q8" s="5">
+        <f t="shared" si="2"/>
         <v>3.3584874367692183</v>
       </c>
       <c r="R8" s="5">
-        <v>0</v>
+        <v>3.3584874367692183</v>
       </c>
       <c r="S8" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T8" s="5">
+        <f t="shared" si="3"/>
         <v>3.55750891450369</v>
       </c>
-      <c r="T8" s="5">
+      <c r="U8" s="5">
         <v>3.225806451612903</v>
       </c>
-      <c r="U8" s="5">
+      <c r="V8" s="5">
         <v>0.33170246289078698</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -7706,23 +7745,27 @@
         <v>1.0991594004992109</v>
       </c>
       <c r="Q9" s="5">
+        <f t="shared" si="2"/>
+        <v>36.102125563850862</v>
+      </c>
+      <c r="R9" s="5">
         <v>36.051756752219028</v>
       </c>
-      <c r="R9" s="5">
+      <c r="S9" s="5">
         <v>5.0368811631837568E-2</v>
       </c>
-      <c r="S9" s="5">
-        <f t="shared" si="2"/>
+      <c r="T9" s="5">
+        <f t="shared" si="3"/>
         <v>5.7767430407091931</v>
       </c>
-      <c r="T9" s="5">
+      <c r="U9" s="5">
         <v>4.2108326524216206</v>
       </c>
-      <c r="U9" s="5">
+      <c r="V9" s="5">
         <v>1.5659103882875725</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -7774,23 +7817,27 @@
         <v>0</v>
       </c>
       <c r="Q10" s="5">
+        <f t="shared" si="2"/>
         <v>9.4634238667549928E-2</v>
       </c>
       <c r="R10" s="5">
-        <v>0</v>
+        <v>9.4634238667549928E-2</v>
       </c>
       <c r="S10" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T10" s="5">
+        <f t="shared" si="3"/>
         <v>0.28390271600264977</v>
       </c>
-      <c r="T10" s="5">
+      <c r="U10" s="5">
         <v>0.28390271600264977</v>
       </c>
-      <c r="U10" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V10" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -7842,23 +7889,27 @@
         <v>8.8295023103864383E-3</v>
       </c>
       <c r="Q11" s="5">
+        <f t="shared" si="2"/>
         <v>8.5351855667068904E-2</v>
       </c>
       <c r="R11" s="5">
-        <v>0</v>
+        <v>8.5351855667068904E-2</v>
       </c>
       <c r="S11" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T11" s="5">
+        <f t="shared" si="3"/>
         <v>0.22073755775966095</v>
       </c>
-      <c r="T11" s="5">
+      <c r="U11" s="5">
         <v>0.22073755775966095</v>
       </c>
-      <c r="U11" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V11" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -7910,23 +7961,27 @@
         <v>0.55498061394047171</v>
       </c>
       <c r="Q12" s="5">
+        <f t="shared" si="2"/>
         <v>0.57484039296854506</v>
       </c>
       <c r="R12" s="5">
-        <v>0</v>
+        <v>0.57484039296854506</v>
       </c>
       <c r="S12" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T12" s="5">
+        <f t="shared" si="3"/>
         <v>1.5587193539923623</v>
       </c>
-      <c r="T12" s="5">
+      <c r="U12" s="5">
         <v>1.4209762994490278</v>
       </c>
-      <c r="U12" s="5">
+      <c r="V12" s="5">
         <v>0.13774305454333441</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -7978,23 +8033,27 @@
         <v>0.30155353921542227</v>
       </c>
       <c r="Q13" s="5">
+        <f t="shared" si="2"/>
         <v>0.93158504079050108</v>
       </c>
       <c r="R13" s="5">
-        <v>0</v>
+        <v>0.93158504079050108</v>
       </c>
       <c r="S13" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T13" s="5">
+        <f t="shared" si="3"/>
         <v>1.9412509086992813</v>
       </c>
-      <c r="T13" s="5">
+      <c r="U13" s="5">
         <v>1.4269944266444092</v>
       </c>
-      <c r="U13" s="5">
+      <c r="V13" s="5">
         <v>0.51425648205487196</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -8046,23 +8105,27 @@
         <v>0.5250875145857643</v>
       </c>
       <c r="Q14" s="5">
+        <f t="shared" si="2"/>
         <v>0.12252042007001165</v>
       </c>
       <c r="R14" s="5">
-        <v>0</v>
+        <v>0.12252042007001165</v>
       </c>
       <c r="S14" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T14" s="5">
+        <f t="shared" si="3"/>
         <v>7.0011668611435235E-2</v>
       </c>
-      <c r="T14" s="5">
+      <c r="U14" s="5">
         <v>7.0011668611435235E-2</v>
       </c>
-      <c r="U14" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V14" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -8114,23 +8177,27 @@
         <v>1.2299517858899931E-2</v>
       </c>
       <c r="Q15" s="5">
+        <f t="shared" si="2"/>
         <v>0.28042900718291841</v>
       </c>
       <c r="R15" s="5">
-        <v>0</v>
+        <v>0.28042900718291841</v>
       </c>
       <c r="S15" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T15" s="5">
+        <f t="shared" si="3"/>
         <v>2.2483518646069074</v>
       </c>
-      <c r="T15" s="5">
+      <c r="U15" s="5">
         <v>1.6112368395158911</v>
       </c>
-      <c r="U15" s="5">
+      <c r="V15" s="5">
         <v>0.63711502509101636</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -8182,23 +8249,27 @@
         <v>3.7854207224745834E-2</v>
       </c>
       <c r="Q16" s="5">
+        <f t="shared" si="2"/>
         <v>5.4077438892494049E-2</v>
       </c>
       <c r="R16" s="5">
-        <v>0</v>
+        <v>5.4077438892494049E-2</v>
       </c>
       <c r="S16" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T16" s="5">
+        <f t="shared" si="3"/>
         <v>0.79493835171966254</v>
       </c>
-      <c r="T16" s="5">
+      <c r="U16" s="5">
         <v>0.68678347393467443</v>
       </c>
-      <c r="U16" s="5">
+      <c r="V16" s="5">
         <v>0.1081548777849881</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -8250,23 +8321,27 @@
         <v>0.47272899696677534</v>
       </c>
       <c r="Q17" s="5">
+        <f t="shared" si="2"/>
+        <v>1.753264200908387</v>
+      </c>
+      <c r="R17" s="5">
         <v>1.7183483509804458</v>
       </c>
-      <c r="R17" s="5">
+      <c r="S17" s="5">
         <v>3.4915849927941153E-2</v>
       </c>
-      <c r="S17" s="5">
-        <f t="shared" si="2"/>
+      <c r="T17" s="5">
+        <f t="shared" si="3"/>
         <v>3.3254832540422643</v>
       </c>
-      <c r="T17" s="5">
+      <c r="U17" s="5">
         <v>2.4883649755229835</v>
       </c>
-      <c r="U17" s="5">
+      <c r="V17" s="5">
         <v>0.83711827851928067</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>33</v>
       </c>
@@ -8318,23 +8393,27 @@
         <v>1.1851149561507466E-2</v>
       </c>
       <c r="Q18" s="5">
+        <f t="shared" si="2"/>
         <v>0.40293908509125381</v>
       </c>
       <c r="R18" s="5">
-        <v>0</v>
+        <v>0.40293908509125381</v>
       </c>
       <c r="S18" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T18" s="5">
+        <f t="shared" si="3"/>
         <v>1.3273287508888363</v>
       </c>
-      <c r="T18" s="5">
+      <c r="U18" s="5">
         <v>0.97179426404361224</v>
       </c>
-      <c r="U18" s="5">
+      <c r="V18" s="5">
         <v>0.35553448684522398</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>34</v>
       </c>
@@ -8386,23 +8465,27 @@
         <v>0.1513736807854455</v>
       </c>
       <c r="Q19" s="5">
+        <f t="shared" si="2"/>
         <v>0.27162380103556577</v>
       </c>
       <c r="R19" s="5">
-        <v>0</v>
+        <v>0.27162380103556577</v>
       </c>
       <c r="S19" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T19" s="5">
+        <f t="shared" si="3"/>
         <v>3.6980448745154626</v>
       </c>
-      <c r="T19" s="5">
+      <c r="U19" s="5">
         <v>3.2821209291797526</v>
       </c>
-      <c r="U19" s="5">
+      <c r="V19" s="5">
         <v>0.41592394533571003</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -8454,23 +8537,27 @@
         <v>7.4174053672831627E-2</v>
       </c>
       <c r="Q20" s="5">
+        <f t="shared" si="2"/>
         <v>8.5117766509806778E-2</v>
       </c>
       <c r="R20" s="5">
-        <v>0</v>
+        <v>8.5117766509806778E-2</v>
       </c>
       <c r="S20" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T20" s="5">
+        <f t="shared" si="3"/>
         <v>4.2583202616763334</v>
       </c>
-      <c r="T20" s="5">
+      <c r="U20" s="5">
         <v>3.1043665414219532</v>
       </c>
-      <c r="U20" s="5">
+      <c r="V20" s="5">
         <v>1.1539537202543806</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -8522,23 +8609,27 @@
         <v>0.2263802263802264</v>
       </c>
       <c r="Q21" s="5">
+        <f t="shared" si="2"/>
         <v>0.27951027951027951</v>
       </c>
       <c r="R21" s="5">
-        <v>0</v>
+        <v>0.27951027951027951</v>
       </c>
       <c r="S21" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T21" s="5">
+        <f t="shared" si="3"/>
         <v>3.0399630399630402</v>
       </c>
-      <c r="T21" s="5">
+      <c r="U21" s="5">
         <v>2.9106029106029108</v>
       </c>
-      <c r="U21" s="5">
+      <c r="V21" s="5">
         <v>0.12936012936012936</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>37</v>
       </c>
@@ -8590,23 +8681,27 @@
         <v>0.4356790546201651</v>
       </c>
       <c r="Q22" s="5">
+        <f t="shared" si="2"/>
         <v>1.6305179335115878</v>
       </c>
       <c r="R22" s="5">
-        <v>0</v>
+        <v>1.6305179335115878</v>
       </c>
       <c r="S22" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T22" s="5">
+        <f t="shared" si="3"/>
         <v>5.7942400023313931</v>
       </c>
-      <c r="T22" s="5">
+      <c r="U22" s="5">
         <v>4.4099754475181596</v>
       </c>
-      <c r="U22" s="5">
+      <c r="V22" s="5">
         <v>1.3842645548132335</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>38</v>
       </c>
@@ -8658,23 +8753,27 @@
         <v>0.77008114944023653</v>
       </c>
       <c r="Q23" s="5">
+        <f t="shared" si="2"/>
         <v>1.7684485774034233</v>
       </c>
       <c r="R23" s="5">
-        <v>0</v>
+        <v>1.7684485774034233</v>
       </c>
       <c r="S23" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T23" s="5">
+        <f t="shared" si="3"/>
         <v>2.2630118044883751</v>
       </c>
-      <c r="T23" s="5">
+      <c r="U23" s="5">
         <v>1.5969771747947306</v>
       </c>
-      <c r="U23" s="5">
+      <c r="V23" s="5">
         <v>0.66603462969364458</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>39</v>
       </c>
@@ -8726,23 +8825,27 @@
         <v>0</v>
       </c>
       <c r="Q24" s="5">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R24" s="5">
         <v>0</v>
       </c>
       <c r="S24" s="5">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="T24" s="5">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="U24" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V24" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>40</v>
       </c>
@@ -8794,23 +8897,27 @@
         <v>1.2027395388980993</v>
       </c>
       <c r="Q25" s="5">
+        <f t="shared" si="2"/>
         <v>2.7153226657725291</v>
       </c>
       <c r="R25" s="5">
-        <v>0</v>
+        <v>2.7153226657725291</v>
       </c>
       <c r="S25" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T25" s="5">
+        <f t="shared" si="3"/>
         <v>1.4579413718806078</v>
       </c>
-      <c r="T25" s="5">
+      <c r="U25" s="5">
         <v>1.3213369843960534</v>
       </c>
-      <c r="U25" s="5">
+      <c r="V25" s="5">
         <v>0.13660438748455439</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>41</v>
       </c>
@@ -8862,23 +8969,27 @@
         <v>1.040949759119064</v>
       </c>
       <c r="Q26" s="5">
+        <f t="shared" si="2"/>
         <v>0.25808671713695802</v>
       </c>
       <c r="R26" s="5">
-        <v>0</v>
+        <v>0.25808671713695802</v>
       </c>
       <c r="S26" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T26" s="5">
+        <f t="shared" si="3"/>
         <v>4.8778389538885065</v>
       </c>
-      <c r="T26" s="5">
+      <c r="U26" s="5">
         <v>4.6025464556090849</v>
       </c>
-      <c r="U26" s="5">
+      <c r="V26" s="5">
         <v>0.27529249827942187</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>42</v>
       </c>
@@ -8930,23 +9041,27 @@
         <v>1.2747628009856615</v>
       </c>
       <c r="Q27" s="5">
+        <f t="shared" si="2"/>
+        <v>4.8191660684142095</v>
+      </c>
+      <c r="R27" s="5">
         <v>4.7379169172859381</v>
       </c>
-      <c r="R27" s="5">
+      <c r="S27" s="5">
         <v>8.1249151128271788E-2</v>
       </c>
-      <c r="S27" s="5">
-        <f t="shared" si="2"/>
+      <c r="T27" s="5">
+        <f t="shared" si="3"/>
         <v>2.319198406384809</v>
       </c>
-      <c r="T27" s="5">
+      <c r="U27" s="5">
         <v>1.8097136796083224</v>
       </c>
-      <c r="U27" s="5">
+      <c r="V27" s="5">
         <v>0.50948472677648649</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>43</v>
       </c>
@@ -8998,23 +9113,27 @@
         <v>0.62725109994186556</v>
       </c>
       <c r="Q28" s="5">
+        <f t="shared" si="2"/>
+        <v>2.3436108983806023</v>
+      </c>
+      <c r="R28" s="5">
         <v>2.2998491937334955</v>
       </c>
-      <c r="R28" s="5">
+      <c r="S28" s="5">
         <v>4.3761704647106901E-2</v>
       </c>
-      <c r="S28" s="5">
-        <f t="shared" si="2"/>
+      <c r="T28" s="5">
+        <f t="shared" si="3"/>
         <v>3.2179869186826009</v>
       </c>
-      <c r="T28" s="5">
+      <c r="U28" s="5">
         <v>2.3221590823771185</v>
       </c>
-      <c r="U28" s="5">
+      <c r="V28" s="5">
         <v>0.89582783630548246</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>44</v>
       </c>
@@ -9066,23 +9185,27 @@
         <v>1.1851149561507466E-2</v>
       </c>
       <c r="Q29" s="5">
+        <f t="shared" si="2"/>
         <v>0.40293908509125381</v>
       </c>
       <c r="R29" s="5">
-        <v>0</v>
+        <v>0.40293908509125381</v>
       </c>
       <c r="S29" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T29" s="5">
+        <f t="shared" si="3"/>
         <v>1.3273287508888363</v>
       </c>
-      <c r="T29" s="5">
+      <c r="U29" s="5">
         <v>0.97179426404361224</v>
       </c>
-      <c r="U29" s="5">
+      <c r="V29" s="5">
         <v>0.35553448684522398</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>45</v>
       </c>
@@ -9134,23 +9257,27 @@
         <v>0.4325622441155621</v>
       </c>
       <c r="Q30" s="5">
+        <f t="shared" si="2"/>
         <v>1.6268101789563532</v>
       </c>
       <c r="R30" s="5">
-        <v>0</v>
+        <v>1.6268101789563532</v>
       </c>
       <c r="S30" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T30" s="5">
+        <f t="shared" si="3"/>
         <v>5.7752123027067688</v>
       </c>
-      <c r="T30" s="5">
+      <c r="U30" s="5">
         <v>4.3820436034315637</v>
       </c>
-      <c r="U30" s="5">
+      <c r="V30" s="5">
         <v>1.393168699275205</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>46</v>
       </c>
@@ -9202,23 +9329,27 @@
         <v>0.27430093209054596</v>
       </c>
       <c r="Q31" s="5">
+        <f t="shared" si="2"/>
+        <v>3.9840213049267645</v>
+      </c>
+      <c r="R31" s="5">
         <v>3.6697736351531294</v>
       </c>
-      <c r="R31" s="5">
+      <c r="S31" s="5">
         <v>0.31424766977363516</v>
       </c>
-      <c r="S31" s="5">
-        <f t="shared" si="2"/>
+      <c r="T31" s="5">
+        <f t="shared" si="3"/>
         <v>5.3581890812250332</v>
       </c>
-      <c r="T31" s="5">
+      <c r="U31" s="5">
         <v>1.0998668442077231</v>
       </c>
-      <c r="U31" s="5">
+      <c r="V31" s="5">
         <v>4.2583222370173104</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>47</v>
       </c>
@@ -9270,23 +9401,27 @@
         <v>1.4328867192909569</v>
       </c>
       <c r="Q32" s="5">
+        <f t="shared" si="2"/>
+        <v>5.0642224068688551</v>
+      </c>
+      <c r="R32" s="5">
         <v>4.9953044938374189</v>
       </c>
-      <c r="R32" s="5">
+      <c r="S32" s="5">
         <v>6.8917913031436087E-2</v>
       </c>
-      <c r="S32" s="5">
-        <f t="shared" si="2"/>
+      <c r="T32" s="5">
+        <f t="shared" si="3"/>
         <v>1.579810621797535</v>
       </c>
-      <c r="T32" s="5">
+      <c r="U32" s="5">
         <v>1.3309704334579697</v>
       </c>
-      <c r="U32" s="5">
+      <c r="V32" s="5">
         <v>0.24884018833956517</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>48</v>
       </c>
@@ -9338,23 +9473,27 @@
         <v>1.0434134525805852</v>
       </c>
       <c r="Q33" s="5">
+        <f t="shared" si="2"/>
         <v>2.6701240088607334</v>
       </c>
       <c r="R33" s="5">
-        <v>0</v>
+        <v>2.6701240088607334</v>
       </c>
       <c r="S33" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T33" s="5">
+        <f t="shared" si="3"/>
         <v>4.525081257892885</v>
       </c>
-      <c r="T33" s="5">
+      <c r="U33" s="5">
         <v>4.1136161315032194</v>
       </c>
-      <c r="U33" s="5">
+      <c r="V33" s="5">
         <v>0.41146512638966526</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>49</v>
       </c>
@@ -9406,23 +9545,27 @@
         <v>2.2060445621001543E-2</v>
       </c>
       <c r="Q34" s="5">
+        <f t="shared" si="2"/>
         <v>3.0884623869402161E-2</v>
       </c>
       <c r="R34" s="5">
-        <v>0</v>
+        <v>3.0884623869402161E-2</v>
       </c>
       <c r="S34" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T34" s="5">
+        <f t="shared" si="3"/>
         <v>0.16765938671961172</v>
       </c>
-      <c r="T34" s="5">
+      <c r="U34" s="5">
         <v>0.16765938671961172</v>
       </c>
-      <c r="U34" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V34" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>50</v>
       </c>
@@ -9474,23 +9617,27 @@
         <v>0.60332341559616209</v>
       </c>
       <c r="Q35" s="5">
+        <f t="shared" si="2"/>
         <v>0.49776699830988869</v>
       </c>
       <c r="R35" s="5">
-        <v>0</v>
+        <v>0.49776699830988869</v>
       </c>
       <c r="S35" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T35" s="5">
+        <f t="shared" si="3"/>
         <v>1.5627990177612774</v>
       </c>
-      <c r="T35" s="5">
+      <c r="U35" s="5">
         <v>1.4169538915871134</v>
       </c>
-      <c r="U35" s="5">
+      <c r="V35" s="5">
         <v>0.14584512617416406</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>51</v>
       </c>
@@ -9542,23 +9689,27 @@
         <v>1.3449899125756557E-2</v>
       </c>
       <c r="Q36" s="5">
+        <f t="shared" si="2"/>
         <v>0.43039677202420984</v>
       </c>
       <c r="R36" s="5">
-        <v>0</v>
+        <v>0.43039677202420984</v>
       </c>
       <c r="S36" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T36" s="5">
+        <f t="shared" si="3"/>
         <v>0.4438466711499664</v>
       </c>
-      <c r="T36" s="5">
+      <c r="U36" s="5">
         <v>0.4438466711499664</v>
       </c>
-      <c r="U36" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V36" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>52</v>
       </c>
@@ -9610,23 +9761,27 @@
         <v>0</v>
       </c>
       <c r="Q37" s="5">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R37" s="5">
         <v>0</v>
       </c>
       <c r="S37" s="5">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="T37" s="5">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="U37" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V37" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>53</v>
       </c>
@@ -9678,23 +9833,27 @@
         <v>0.11574074074074073</v>
       </c>
       <c r="Q38" s="5">
-        <v>0.19290123456790123</v>
-      </c>
-      <c r="R38" s="5">
-        <v>0</v>
-      </c>
-      <c r="S38" s="5">
         <f t="shared" si="2"/>
         <v>0.19290123456790123</v>
       </c>
+      <c r="R38" s="5">
+        <v>0.19290123456790123</v>
+      </c>
+      <c r="S38" s="5">
+        <v>0</v>
+      </c>
       <c r="T38" s="5">
+        <f t="shared" si="3"/>
         <v>0.19290123456790123</v>
       </c>
       <c r="U38" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
+        <v>0.19290123456790123</v>
+      </c>
+      <c r="V38" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>54</v>
       </c>
@@ -9746,23 +9905,27 @@
         <v>0</v>
       </c>
       <c r="Q39" s="5">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R39" s="5">
         <v>0</v>
       </c>
       <c r="S39" s="5">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="T39" s="5">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="U39" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V39" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>55</v>
       </c>
@@ -9814,23 +9977,27 @@
         <v>1.3954674943662571</v>
       </c>
       <c r="Q40" s="5">
+        <f t="shared" si="2"/>
         <v>3.6566180534886685</v>
       </c>
       <c r="R40" s="5">
-        <v>0</v>
+        <v>3.6566180534886685</v>
       </c>
       <c r="S40" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T40" s="5">
+        <f t="shared" si="3"/>
         <v>1.3733577107870232</v>
       </c>
-      <c r="T40" s="5">
+      <c r="U40" s="5">
         <v>1.2372975041455843</v>
       </c>
-      <c r="U40" s="5">
+      <c r="V40" s="5">
         <v>0.13606020664143884</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>56</v>
       </c>
@@ -9882,23 +10049,27 @@
         <v>1.0663611527275931</v>
       </c>
       <c r="Q41" s="5">
+        <f t="shared" si="2"/>
         <v>0.25557416057107607</v>
       </c>
       <c r="R41" s="5">
-        <v>0</v>
+        <v>0.25557416057107607</v>
       </c>
       <c r="S41" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T41" s="5">
+        <f t="shared" si="3"/>
         <v>4.9352251696483647</v>
       </c>
-      <c r="T41" s="5">
+      <c r="U41" s="5">
         <v>4.6532123028113155</v>
       </c>
-      <c r="U41" s="5">
+      <c r="V41" s="5">
         <v>0.2820128668370494</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>57</v>
       </c>
@@ -9950,23 +10121,27 @@
         <v>0.14889815366289458</v>
       </c>
       <c r="Q42" s="5">
+        <f t="shared" si="2"/>
         <v>0.2441929720071471</v>
       </c>
       <c r="R42" s="5">
-        <v>0</v>
+        <v>0.2441929720071471</v>
       </c>
       <c r="S42" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T42" s="5">
+        <f t="shared" si="3"/>
         <v>3.0315664085765337</v>
       </c>
-      <c r="T42" s="5">
+      <c r="U42" s="5">
         <v>2.5610482430017867</v>
       </c>
-      <c r="U42" s="5">
+      <c r="V42" s="5">
         <v>0.47051816557474685</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>58</v>
       </c>
@@ -10018,23 +10193,27 @@
         <v>9.4410876132930519E-2</v>
       </c>
       <c r="Q43" s="5">
+        <f t="shared" si="2"/>
         <v>0.16993957703927492</v>
       </c>
       <c r="R43" s="5">
-        <v>0</v>
+        <v>0.16993957703927492</v>
       </c>
       <c r="S43" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T43" s="5">
+        <f t="shared" si="3"/>
         <v>2.5490936555891239</v>
       </c>
-      <c r="T43" s="5">
+      <c r="U43" s="5">
         <v>2.3980362537764353</v>
       </c>
-      <c r="U43" s="5">
+      <c r="V43" s="5">
         <v>0.15105740181268881</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>59</v>
       </c>
@@ -10086,23 +10265,27 @@
         <v>0.13815971262779772</v>
       </c>
       <c r="Q44" s="5">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R44" s="5">
         <v>0</v>
       </c>
       <c r="S44" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T44" s="5">
+        <f t="shared" si="3"/>
         <v>3.4816247582205029</v>
       </c>
-      <c r="T44" s="5">
+      <c r="U44" s="5">
         <v>3.4263608731693838</v>
       </c>
-      <c r="U44" s="5">
+      <c r="V44" s="5">
         <v>5.5263885051119094E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>60</v>
       </c>
@@ -10154,23 +10337,27 @@
         <v>0</v>
       </c>
       <c r="Q45" s="5">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R45" s="5">
         <v>0</v>
       </c>
       <c r="S45" s="5">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="T45" s="5">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="U45" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V45" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>61</v>
       </c>
@@ -10222,23 +10409,27 @@
         <v>0.40288735940909853</v>
       </c>
       <c r="Q46" s="5">
+        <f t="shared" si="2"/>
         <v>0.75541379889205984</v>
       </c>
       <c r="R46" s="5">
-        <v>0</v>
+        <v>0.75541379889205984</v>
       </c>
       <c r="S46" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T46" s="5">
+        <f t="shared" si="3"/>
         <v>5.346650998824912</v>
       </c>
-      <c r="T46" s="5">
+      <c r="U46" s="5">
         <v>4.7758939063286894</v>
       </c>
-      <c r="U46" s="5">
+      <c r="V46" s="5">
         <v>0.57075709249622297</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>62</v>
       </c>
@@ -10290,23 +10481,27 @@
         <v>2.3926644061320981</v>
       </c>
       <c r="Q47" s="5">
+        <f t="shared" si="2"/>
+        <v>18.300778451693013</v>
+      </c>
+      <c r="R47" s="5">
         <v>17.312192559339032</v>
       </c>
-      <c r="R47" s="5">
+      <c r="S47" s="5">
         <v>0.98858589235398064</v>
       </c>
-      <c r="S47" s="5">
-        <f t="shared" si="2"/>
+      <c r="T47" s="5">
+        <f t="shared" si="3"/>
         <v>1.9532928984192177</v>
       </c>
-      <c r="T47" s="5">
+      <c r="U47" s="5">
         <v>1.1939443144371746</v>
       </c>
-      <c r="U47" s="5">
+      <c r="V47" s="5">
         <v>0.75934858398204308</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>63</v>
       </c>
@@ -10358,23 +10553,27 @@
         <v>1.4723086575450115</v>
       </c>
       <c r="Q48" s="5">
+        <f t="shared" si="2"/>
+        <v>0.68646898151375535</v>
+      </c>
+      <c r="R48" s="5">
         <v>0.61472942399219233</v>
       </c>
-      <c r="R48" s="5">
+      <c r="S48" s="5">
         <v>7.1739557521563052E-2</v>
       </c>
-      <c r="S48" s="5">
-        <f t="shared" si="2"/>
+      <c r="T48" s="5">
+        <f t="shared" si="3"/>
         <v>0.75770154569594339</v>
       </c>
-      <c r="T48" s="5">
+      <c r="U48" s="5">
         <v>0.69153891490750541</v>
       </c>
-      <c r="U48" s="5">
+      <c r="V48" s="5">
         <v>6.6162630788438023E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>64</v>
       </c>
@@ -10426,23 +10625,27 @@
         <v>0.53923037119747264</v>
       </c>
       <c r="Q49" s="5">
+        <f t="shared" si="2"/>
         <v>1.255480813747651</v>
       </c>
       <c r="R49" s="5">
-        <v>0</v>
+        <v>1.255480813747651</v>
       </c>
       <c r="S49" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T49" s="5">
+        <f t="shared" si="3"/>
         <v>6.9500803398785367</v>
       </c>
-      <c r="T49" s="5">
+      <c r="U49" s="5">
         <v>4.0278874697023337</v>
       </c>
-      <c r="U49" s="5">
+      <c r="V49" s="5">
         <v>2.922192870176203</v>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>65</v>
       </c>
@@ -10494,23 +10697,27 @@
         <v>1.2285012285012284E-2</v>
       </c>
       <c r="Q50" s="5">
+        <f t="shared" si="2"/>
         <v>0.18427518427518427</v>
       </c>
       <c r="R50" s="5">
-        <v>0</v>
+        <v>0.18427518427518427</v>
       </c>
       <c r="S50" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T50" s="5">
+        <f t="shared" si="3"/>
         <v>1.8181818181818181</v>
       </c>
-      <c r="T50" s="5">
+      <c r="U50" s="5">
         <v>0.89680589680589673</v>
       </c>
-      <c r="U50" s="5">
+      <c r="V50" s="5">
         <v>0.92137592137592139</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>66</v>
       </c>
@@ -10562,23 +10769,27 @@
         <v>0.14572302909603146</v>
       </c>
       <c r="Q51" s="5">
+        <f t="shared" si="2"/>
         <v>5.9908356406146272E-2</v>
       </c>
       <c r="R51" s="5">
-        <v>0</v>
+        <v>5.9908356406146272E-2</v>
       </c>
       <c r="S51" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T51" s="5">
+        <f t="shared" si="3"/>
         <v>3.0569453214811935</v>
       </c>
-      <c r="T51" s="5">
+      <c r="U51" s="5">
         <v>3.0002752546105147</v>
       </c>
-      <c r="U51" s="5">
+      <c r="V51" s="5">
         <v>5.6670066870678909E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>67</v>
       </c>
@@ -10630,23 +10841,27 @@
         <v>2.3377800803004791</v>
       </c>
       <c r="Q52" s="5">
+        <f t="shared" si="2"/>
         <v>11.358632301515348</v>
       </c>
       <c r="R52" s="5">
-        <v>0</v>
+        <v>11.358632301515348</v>
       </c>
       <c r="S52" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T52" s="5">
+        <f t="shared" si="3"/>
         <v>3.6199974096619609</v>
       </c>
-      <c r="T52" s="5">
+      <c r="U52" s="5">
         <v>2.9573025946552693</v>
       </c>
-      <c r="U52" s="5">
+      <c r="V52" s="5">
         <v>0.6626948150066917</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>68</v>
       </c>
@@ -10698,23 +10913,27 @@
         <v>0.36542023326825851</v>
       </c>
       <c r="Q53" s="5">
+        <f t="shared" si="2"/>
         <v>1.7620263302798218</v>
       </c>
       <c r="R53" s="5">
-        <v>0</v>
+        <v>1.7620263302798218</v>
       </c>
       <c r="S53" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T53" s="5">
+        <f t="shared" si="3"/>
         <v>1.2614506682685089</v>
       </c>
-      <c r="T53" s="5">
+      <c r="U53" s="5">
         <v>1.1813585623466989</v>
       </c>
-      <c r="U53" s="5">
+      <c r="V53" s="5">
         <v>8.0092105921810083E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>69</v>
       </c>
@@ -10766,23 +10985,27 @@
         <v>0</v>
       </c>
       <c r="Q54" s="5">
+        <f t="shared" si="2"/>
         <v>0.24786560176259984</v>
       </c>
       <c r="R54" s="5">
-        <v>0</v>
+        <v>0.24786560176259984</v>
       </c>
       <c r="S54" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T54" s="5">
+        <f t="shared" si="3"/>
         <v>0.89966033232351039</v>
       </c>
-      <c r="T54" s="5">
+      <c r="U54" s="5">
         <v>0.83539888001468821</v>
       </c>
-      <c r="U54" s="5">
+      <c r="V54" s="5">
         <v>6.4261452308822187E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>70</v>
       </c>
@@ -10834,23 +11057,27 @@
         <v>0</v>
       </c>
       <c r="Q55" s="5">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R55" s="5">
         <v>0</v>
       </c>
       <c r="S55" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T55" s="5">
+        <f t="shared" si="3"/>
         <v>0.36611538947102634</v>
       </c>
-      <c r="T55" s="5">
+      <c r="U55" s="5">
         <v>0.36611538947102634</v>
       </c>
-      <c r="U55" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V55" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>71</v>
       </c>
@@ -10902,23 +11129,27 @@
         <v>0.36972527061538957</v>
       </c>
       <c r="Q56" s="5">
+        <f t="shared" si="2"/>
         <v>0.99056452560828345</v>
       </c>
       <c r="R56" s="5">
-        <v>0</v>
+        <v>0.99056452560828345</v>
       </c>
       <c r="S56" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T56" s="5">
+        <f t="shared" si="3"/>
         <v>5.3845249671414681</v>
       </c>
-      <c r="T56" s="5">
+      <c r="U56" s="5">
         <v>4.725217186882233</v>
       </c>
-      <c r="U56" s="5">
+      <c r="V56" s="5">
         <v>0.65930778025923509</v>
       </c>
     </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>72</v>
       </c>
@@ -10970,23 +11201,27 @@
         <v>1.3068153112948586</v>
       </c>
       <c r="Q57" s="5">
+        <f t="shared" si="2"/>
         <v>0.19703272090399288</v>
       </c>
       <c r="R57" s="5">
-        <v>0</v>
+        <v>0.19703272090399288</v>
       </c>
       <c r="S57" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T57" s="5">
+        <f t="shared" si="3"/>
         <v>4.2218891564641892</v>
       </c>
-      <c r="T57" s="5">
+      <c r="U57" s="5">
         <v>4.1595796635287385</v>
       </c>
-      <c r="U57" s="5">
+      <c r="V57" s="5">
         <v>6.2309492935450732E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>73</v>
       </c>
@@ -11038,23 +11273,27 @@
         <v>0.40096401987757796</v>
       </c>
       <c r="Q58" s="5">
+        <f t="shared" si="2"/>
         <v>1.3287265126794208</v>
       </c>
       <c r="R58" s="5">
-        <v>0</v>
+        <v>1.3287265126794208</v>
       </c>
       <c r="S58" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T58" s="5">
+        <f t="shared" si="3"/>
         <v>4.2506451681702817</v>
       </c>
-      <c r="T58" s="5">
+      <c r="U58" s="5">
         <v>4.1120139910849485</v>
       </c>
-      <c r="U58" s="5">
+      <c r="V58" s="5">
         <v>0.13863117708533282</v>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>74</v>
       </c>
@@ -11106,23 +11345,27 @@
         <v>1.2671594508975714E-2</v>
       </c>
       <c r="Q59" s="5">
+        <f t="shared" si="2"/>
         <v>0.24076029567053855</v>
       </c>
       <c r="R59" s="5">
-        <v>0</v>
+        <v>0.24076029567053855</v>
       </c>
       <c r="S59" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T59" s="5">
+        <f t="shared" si="3"/>
         <v>1.8204857444561773</v>
       </c>
-      <c r="T59" s="5">
+      <c r="U59" s="5">
         <v>1.6092925026399154</v>
       </c>
-      <c r="U59" s="5">
+      <c r="V59" s="5">
         <v>0.21119324181626187</v>
       </c>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>75</v>
       </c>
@@ -11174,23 +11417,27 @@
         <v>5.6834327934072178E-2</v>
       </c>
       <c r="Q60" s="5">
+        <f t="shared" si="2"/>
         <v>8.525149190110827E-2</v>
       </c>
       <c r="R60" s="5">
-        <v>0</v>
+        <v>8.525149190110827E-2</v>
       </c>
       <c r="S60" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T60" s="5">
+        <f t="shared" si="3"/>
         <v>4.2503958104981123</v>
       </c>
-      <c r="T60" s="5">
+      <c r="U60" s="5">
         <v>3.1664839848983073</v>
       </c>
-      <c r="U60" s="5">
+      <c r="V60" s="5">
         <v>1.083911825599805</v>
       </c>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>76</v>
       </c>
@@ -11242,23 +11489,27 @@
         <v>2.0836433993153745</v>
       </c>
       <c r="Q61" s="5">
+        <f t="shared" si="2"/>
         <v>0.16371483851763655</v>
       </c>
       <c r="R61" s="5">
-        <v>0</v>
+        <v>0.16371483851763655</v>
       </c>
       <c r="S61" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T61" s="5">
+        <f t="shared" si="3"/>
         <v>6.1765143622562881</v>
       </c>
-      <c r="T61" s="5">
+      <c r="U61" s="5">
         <v>5.6556035124274446</v>
       </c>
-      <c r="U61" s="5">
+      <c r="V61" s="5">
         <v>0.52091084982884361</v>
       </c>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>77</v>
       </c>
@@ -11310,23 +11561,27 @@
         <v>2.0864381520119228</v>
       </c>
       <c r="Q62" s="5">
+        <f t="shared" si="2"/>
         <v>0.16393442622950818</v>
       </c>
       <c r="R62" s="5">
-        <v>0</v>
+        <v>0.16393442622950818</v>
       </c>
       <c r="S62" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T62" s="5">
+        <f t="shared" si="3"/>
         <v>6.1847988077496279</v>
       </c>
-      <c r="T62" s="5">
+      <c r="U62" s="5">
         <v>5.6631892697466473</v>
       </c>
-      <c r="U62" s="5">
+      <c r="V62" s="5">
         <v>0.52160953800298071</v>
       </c>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>78</v>
       </c>
@@ -11378,23 +11633,27 @@
         <v>8.4222346996069619E-2</v>
       </c>
       <c r="Q63" s="5">
+        <f t="shared" si="2"/>
         <v>4.407636159460977</v>
       </c>
       <c r="R63" s="5">
-        <v>0</v>
+        <v>4.407636159460977</v>
       </c>
       <c r="S63" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T63" s="5">
+        <f t="shared" si="3"/>
         <v>2.8542017593112488</v>
       </c>
-      <c r="T63" s="5">
+      <c r="U63" s="5">
         <v>2.0774845592363844</v>
       </c>
-      <c r="U63" s="5">
+      <c r="V63" s="5">
         <v>0.77671720007486433</v>
       </c>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>79</v>
       </c>
@@ -11446,23 +11705,27 @@
         <v>2.0375749723098786</v>
       </c>
       <c r="Q64" s="5">
+        <f t="shared" si="2"/>
         <v>4.1796409688407768E-3</v>
       </c>
       <c r="R64" s="5">
-        <v>0</v>
+        <v>4.1796409688407768E-3</v>
       </c>
       <c r="S64" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T64" s="5">
+        <f t="shared" si="3"/>
         <v>5.901653048003177</v>
       </c>
-      <c r="T64" s="5">
+      <c r="U64" s="5">
         <v>5.8243296900796224</v>
       </c>
-      <c r="U64" s="5">
+      <c r="V64" s="5">
         <v>7.7323357923554367E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>80</v>
       </c>
@@ -11514,23 +11777,27 @@
         <v>1.1176997568363125</v>
       </c>
       <c r="Q65" s="5">
+        <f t="shared" si="2"/>
         <v>0.16637515464357325</v>
       </c>
       <c r="R65" s="5">
-        <v>0</v>
+        <v>0.16637515464357325</v>
       </c>
       <c r="S65" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T65" s="5">
+        <f t="shared" si="3"/>
         <v>4.5689177082888959</v>
       </c>
-      <c r="T65" s="5">
+      <c r="U65" s="5">
         <v>4.2873597542766948</v>
       </c>
-      <c r="U65" s="5">
+      <c r="V65" s="5">
         <v>0.28155795401220085</v>
       </c>
     </row>
-    <row r="66" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>81</v>
       </c>
@@ -11582,23 +11849,27 @@
         <v>0</v>
       </c>
       <c r="Q66" s="5">
+        <f t="shared" si="2"/>
         <v>0.34870819464257413</v>
       </c>
       <c r="R66" s="5">
-        <v>0</v>
+        <v>0.34870819464257413</v>
       </c>
       <c r="S66" s="5">
-        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T66" s="5">
+        <f t="shared" si="3"/>
         <v>0.31700744967506739</v>
       </c>
-      <c r="T66" s="5">
+      <c r="U66" s="5">
         <v>0.31700744967506739</v>
       </c>
-      <c r="U66" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V66" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>82</v>
       </c>
@@ -11612,7 +11883,7 @@
         <v>0</v>
       </c>
       <c r="E67" s="5">
-        <f t="shared" ref="E67:E94" si="3">SUM(F67:I67)</f>
+        <f t="shared" ref="E67:E94" si="4">SUM(F67:I67)</f>
         <v>43.811240290399553</v>
       </c>
       <c r="F67" s="5">
@@ -11631,7 +11902,7 @@
         <v>5.8384525562268363E-2</v>
       </c>
       <c r="K67" s="5">
-        <f t="shared" ref="K67:K94" si="4">SUM(L67:N67)</f>
+        <f t="shared" ref="K67:K94" si="5">SUM(L67:N67)</f>
         <v>46.527389957861601</v>
       </c>
       <c r="L67" s="5">
@@ -11650,23 +11921,27 @@
         <v>0.61938366248667309</v>
       </c>
       <c r="Q67" s="5">
+        <f t="shared" ref="Q67:Q94" si="6">SUM(R67:S67)</f>
         <v>0.32238411940904704</v>
       </c>
       <c r="R67" s="5">
-        <v>0</v>
+        <v>0.32238411940904704</v>
       </c>
       <c r="S67" s="5">
-        <f t="shared" ref="S67:S94" si="5">SUM(T67:U67)</f>
+        <v>0</v>
+      </c>
+      <c r="T67" s="5">
+        <f t="shared" ref="T67:T94" si="7">SUM(U67:V67)</f>
         <v>6.4502208458140835</v>
       </c>
-      <c r="T67" s="5">
+      <c r="U67" s="5">
         <v>5.891760166522821</v>
       </c>
-      <c r="U67" s="5">
+      <c r="V67" s="5">
         <v>0.55846067929126264</v>
       </c>
     </row>
-    <row r="68" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>83</v>
       </c>
@@ -11680,7 +11955,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>89.744995887030456</v>
       </c>
       <c r="F68" s="5">
@@ -11699,7 +11974,7 @@
         <v>5.4839594187003016E-2</v>
       </c>
       <c r="K68" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>8.4178777077049638</v>
       </c>
       <c r="L68" s="5">
@@ -11718,23 +11993,27 @@
         <v>4.1129695640252262E-2</v>
       </c>
       <c r="Q68" s="5">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="R68" s="5">
         <v>0</v>
       </c>
       <c r="S68" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T68" s="5">
+        <f t="shared" si="7"/>
         <v>1.686317521250343</v>
       </c>
-      <c r="T68" s="5">
+      <c r="U68" s="5">
         <v>1.686317521250343</v>
       </c>
-      <c r="U68" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V68" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>84</v>
       </c>
@@ -11748,7 +12027,7 @@
         <v>0</v>
       </c>
       <c r="E69" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>93.967661691542304</v>
       </c>
       <c r="F69" s="5">
@@ -11767,7 +12046,7 @@
         <v>6.2189054726368161E-2</v>
       </c>
       <c r="K69" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>4.8922056384742945</v>
       </c>
       <c r="L69" s="5">
@@ -11786,23 +12065,27 @@
         <v>6.2189054726368161E-2</v>
       </c>
       <c r="Q69" s="5">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="R69" s="5">
         <v>0</v>
       </c>
       <c r="S69" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T69" s="5">
+        <f t="shared" si="7"/>
         <v>0.93283582089552231</v>
       </c>
-      <c r="T69" s="5">
+      <c r="U69" s="5">
         <v>0.93283582089552231</v>
       </c>
-      <c r="U69" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V69" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>85</v>
       </c>
@@ -11816,7 +12099,7 @@
         <v>0</v>
       </c>
       <c r="E70" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>92.905675459632292</v>
       </c>
       <c r="F70" s="5">
@@ -11835,7 +12118,7 @@
         <v>5.9952038369304551E-2</v>
       </c>
       <c r="K70" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>5.8952837729816148</v>
       </c>
       <c r="L70" s="5">
@@ -11854,23 +12137,27 @@
         <v>5.9952038369304551E-2</v>
       </c>
       <c r="Q70" s="5">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="R70" s="5">
         <v>0</v>
       </c>
       <c r="S70" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T70" s="5">
+        <f t="shared" si="7"/>
         <v>0.9992006394884092</v>
       </c>
-      <c r="T70" s="5">
+      <c r="U70" s="5">
         <v>0.9992006394884092</v>
       </c>
-      <c r="U70" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V70" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>86</v>
       </c>
@@ -11884,7 +12171,7 @@
         <v>0</v>
       </c>
       <c r="E71" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>92.002176278563653</v>
       </c>
       <c r="F71" s="5">
@@ -11903,7 +12190,7 @@
         <v>0</v>
       </c>
       <c r="K71" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>5.3862894450489662</v>
       </c>
       <c r="L71" s="5">
@@ -11922,23 +12209,27 @@
         <v>0</v>
       </c>
       <c r="Q71" s="5">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="R71" s="5">
         <v>0</v>
       </c>
       <c r="S71" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T71" s="5">
+        <f t="shared" si="7"/>
         <v>2.6115342763873777</v>
       </c>
-      <c r="T71" s="5">
+      <c r="U71" s="5">
         <v>2.6115342763873777</v>
       </c>
-      <c r="U71" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V71" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>87</v>
       </c>
@@ -11952,7 +12243,7 @@
         <v>0</v>
       </c>
       <c r="E72" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>21.680024348178961</v>
       </c>
       <c r="F72" s="5">
@@ -11971,7 +12262,7 @@
         <v>3.0080146089073754</v>
       </c>
       <c r="K72" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>51.55219640864361</v>
       </c>
       <c r="L72" s="5">
@@ -11990,23 +12281,27 @@
         <v>4.7681850461600899</v>
       </c>
       <c r="Q72" s="5">
+        <f t="shared" si="6"/>
         <v>2.637719387237496</v>
       </c>
       <c r="R72" s="5">
-        <v>0</v>
+        <v>2.637719387237496</v>
       </c>
       <c r="S72" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T72" s="5">
+        <f t="shared" si="7"/>
         <v>8.4508471137262848</v>
       </c>
-      <c r="T72" s="5">
+      <c r="U72" s="5">
         <v>8.1008420411890025</v>
       </c>
-      <c r="U72" s="5">
+      <c r="V72" s="5">
         <v>0.35000507253728314</v>
       </c>
     </row>
-    <row r="73" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>88</v>
       </c>
@@ -12020,7 +12315,7 @@
         <v>0</v>
       </c>
       <c r="E73" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>11.571458464113832</v>
       </c>
       <c r="F73" s="5">
@@ -12039,7 +12334,7 @@
         <v>0.59635907093534213</v>
       </c>
       <c r="K73" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>60.451977401129938</v>
       </c>
       <c r="L73" s="5">
@@ -12058,23 +12353,27 @@
         <v>1.3391922996442771</v>
       </c>
       <c r="Q73" s="5">
+        <f t="shared" si="6"/>
         <v>1.360117179326219</v>
       </c>
       <c r="R73" s="5">
-        <v>0</v>
+        <v>1.360117179326219</v>
       </c>
       <c r="S73" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T73" s="5">
+        <f t="shared" si="7"/>
         <v>5.2939945595312823</v>
       </c>
-      <c r="T73" s="5">
+      <c r="U73" s="5">
         <v>5.1161330822347768</v>
       </c>
-      <c r="U73" s="5">
+      <c r="V73" s="5">
         <v>0.17786147729650553</v>
       </c>
     </row>
-    <row r="74" spans="1:21" ht="27" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:22" ht="27" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>89</v>
       </c>
@@ -12088,7 +12387,7 @@
         <v>0.231327613158435</v>
       </c>
       <c r="E74" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.2078635126427248</v>
       </c>
       <c r="F74" s="5">
@@ -12107,7 +12406,7 @@
         <v>4.3620907300236</v>
       </c>
       <c r="K74" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>82.602862526756155</v>
       </c>
       <c r="L74" s="5">
@@ -12126,23 +12425,27 @@
         <v>2.6230681196805321</v>
       </c>
       <c r="Q74" s="5">
+        <f t="shared" si="6"/>
         <v>5.8543367829199722E-2</v>
       </c>
       <c r="R74" s="5">
-        <v>0</v>
+        <v>5.8543367829199722E-2</v>
       </c>
       <c r="S74" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T74" s="5">
+        <f t="shared" si="7"/>
         <v>0.40065617358108557</v>
       </c>
-      <c r="T74" s="5">
+      <c r="U74" s="5">
         <v>0.37158776524922599</v>
       </c>
-      <c r="U74" s="5">
+      <c r="V74" s="5">
         <v>2.9068408331859589E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>90</v>
       </c>
@@ -12156,7 +12459,7 @@
         <v>0</v>
       </c>
       <c r="E75" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>59.866570737131276</v>
       </c>
       <c r="F75" s="5">
@@ -12175,7 +12478,7 @@
         <v>2.9432925632807902E-2</v>
       </c>
       <c r="K75" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>32.873307606776109</v>
       </c>
       <c r="L75" s="5">
@@ -12194,23 +12497,27 @@
         <v>9.8109752109359669E-2</v>
       </c>
       <c r="Q75" s="5">
+        <f t="shared" si="6"/>
         <v>0.30086990646870299</v>
       </c>
       <c r="R75" s="5">
-        <v>0</v>
+        <v>0.30086990646870299</v>
       </c>
       <c r="S75" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T75" s="5">
+        <f t="shared" si="7"/>
         <v>4.7812152527961276</v>
       </c>
-      <c r="T75" s="5">
+      <c r="U75" s="5">
         <v>4.2383412911243372</v>
       </c>
-      <c r="U75" s="5">
+      <c r="V75" s="5">
         <v>0.54287396167179014</v>
       </c>
     </row>
-    <row r="76" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>91</v>
       </c>
@@ -12224,7 +12531,7 @@
         <v>0</v>
       </c>
       <c r="E76" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>59.90123620455374</v>
       </c>
       <c r="F76" s="5">
@@ -12243,7 +12550,7 @@
         <v>2.9827991913299972E-2</v>
       </c>
       <c r="K76" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>33.069300367878569</v>
       </c>
       <c r="L76" s="5">
@@ -12262,23 +12569,27 @@
         <v>9.9426639710999895E-2</v>
       </c>
       <c r="Q76" s="5">
+        <f t="shared" si="6"/>
         <v>0.30490836178039971</v>
       </c>
       <c r="R76" s="5">
-        <v>0</v>
+        <v>0.30490836178039971</v>
       </c>
       <c r="S76" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T76" s="5">
+        <f t="shared" si="7"/>
         <v>4.5172836642030951</v>
       </c>
-      <c r="T76" s="5">
+      <c r="U76" s="5">
         <v>3.9671229244688959</v>
       </c>
-      <c r="U76" s="5">
+      <c r="V76" s="5">
         <v>0.55016073973419943</v>
       </c>
     </row>
-    <row r="77" spans="1:21" ht="27" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:22" ht="27" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>92</v>
       </c>
@@ -12292,7 +12603,7 @@
         <v>0</v>
       </c>
       <c r="E77" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.4068406446108761</v>
       </c>
       <c r="F77" s="5">
@@ -12311,7 +12622,7 @@
         <v>0.74523437789789948</v>
       </c>
       <c r="K77" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>81.16681447710512</v>
       </c>
       <c r="L77" s="5">
@@ -12330,23 +12641,27 @@
         <v>3.5390202697006585</v>
       </c>
       <c r="Q77" s="5">
+        <f t="shared" si="6"/>
         <v>6.3732713765928956E-2</v>
       </c>
       <c r="R77" s="5">
-        <v>0</v>
+        <v>6.3732713765928956E-2</v>
       </c>
       <c r="S77" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T77" s="5">
+        <f t="shared" si="7"/>
         <v>1.0804212428890816</v>
       </c>
-      <c r="T77" s="5">
+      <c r="U77" s="5">
         <v>1.0568165340868856</v>
       </c>
-      <c r="U77" s="5">
+      <c r="V77" s="5">
         <v>2.3604708802195912E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>93</v>
       </c>
@@ -12360,7 +12675,7 @@
         <v>0</v>
       </c>
       <c r="E78" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>24.756537728139467</v>
       </c>
       <c r="F78" s="5">
@@ -12379,7 +12694,7 @@
         <v>8.3424135113048206E-2</v>
       </c>
       <c r="K78" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>58.691432852083899</v>
       </c>
       <c r="L78" s="5">
@@ -12398,23 +12713,27 @@
         <v>0.89723508580768185</v>
       </c>
       <c r="Q78" s="5">
+        <f t="shared" si="6"/>
+        <v>8.0138245709615923</v>
+      </c>
+      <c r="R78" s="5">
         <v>7.8197357668210303</v>
       </c>
-      <c r="R78" s="5">
+      <c r="S78" s="5">
         <v>0.19408880414056115</v>
       </c>
-      <c r="S78" s="5">
-        <f t="shared" si="5"/>
+      <c r="T78" s="5">
+        <f t="shared" si="7"/>
         <v>5.7392399891037869</v>
       </c>
-      <c r="T78" s="5">
+      <c r="U78" s="5">
         <v>3.1667120675565243</v>
       </c>
-      <c r="U78" s="5">
+      <c r="V78" s="5">
         <v>2.5725279215472621</v>
       </c>
     </row>
-    <row r="79" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>94</v>
       </c>
@@ -12428,7 +12747,7 @@
         <v>0</v>
       </c>
       <c r="E79" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>6.4085045029535497</v>
       </c>
       <c r="F79" s="5">
@@ -12447,7 +12766,7 @@
         <v>0.10544550726820819</v>
       </c>
       <c r="K79" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>86.437340621267708</v>
       </c>
       <c r="L79" s="5">
@@ -12466,23 +12785,27 @@
         <v>2.977221618480939</v>
       </c>
       <c r="Q79" s="5">
+        <f t="shared" si="6"/>
         <v>5.0570804506181476E-2</v>
       </c>
       <c r="R79" s="5">
-        <v>0</v>
+        <v>5.0570804506181476E-2</v>
       </c>
       <c r="S79" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T79" s="5">
+        <f t="shared" si="7"/>
         <v>0.69185164462712112</v>
       </c>
-      <c r="T79" s="5">
+      <c r="U79" s="5">
         <v>0.69077567006315976</v>
       </c>
-      <c r="U79" s="5">
+      <c r="V79" s="5">
         <v>1.0759745639613079E-3</v>
       </c>
     </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>95</v>
       </c>
@@ -12496,7 +12819,7 @@
         <v>0</v>
       </c>
       <c r="E80" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>64.966685347780057</v>
       </c>
       <c r="F80" s="5">
@@ -12515,7 +12838,7 @@
         <v>7.4724453577433209E-2</v>
       </c>
       <c r="K80" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>29.117628744006481</v>
       </c>
       <c r="L80" s="5">
@@ -12534,23 +12857,27 @@
         <v>0.39230338128152442</v>
       </c>
       <c r="Q80" s="5">
+        <f t="shared" si="6"/>
         <v>0.18681113394358304</v>
       </c>
       <c r="R80" s="5">
-        <v>0</v>
+        <v>0.18681113394358304</v>
       </c>
       <c r="S80" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T80" s="5">
+        <f t="shared" si="7"/>
         <v>4.5332835170309487</v>
       </c>
-      <c r="T80" s="5">
+      <c r="U80" s="5">
         <v>4.4585590634535155</v>
       </c>
-      <c r="U80" s="5">
+      <c r="V80" s="5">
         <v>7.4724453577433209E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>96</v>
       </c>
@@ -12564,7 +12891,7 @@
         <v>0</v>
       </c>
       <c r="E81" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>57.407339246935848</v>
       </c>
       <c r="F81" s="5">
@@ -12583,7 +12910,7 @@
         <v>4.7848651036107331E-2</v>
       </c>
       <c r="K81" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>34.528322720747909</v>
       </c>
       <c r="L81" s="5">
@@ -12602,23 +12929,27 @@
         <v>0.43063785932496601</v>
       </c>
       <c r="Q81" s="5">
+        <f t="shared" si="6"/>
         <v>0.59626780521918366</v>
       </c>
       <c r="R81" s="5">
-        <v>0</v>
+        <v>0.59626780521918366</v>
       </c>
       <c r="S81" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T81" s="5">
+        <f t="shared" si="7"/>
         <v>5.9001067392984652</v>
       </c>
-      <c r="T81" s="5">
+      <c r="U81" s="5">
         <v>4.4462438808936655</v>
       </c>
-      <c r="U81" s="5">
+      <c r="V81" s="5">
         <v>1.4538628584047995</v>
       </c>
     </row>
-    <row r="82" spans="1:21" ht="27" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:22" ht="27" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>97</v>
       </c>
@@ -12632,7 +12963,7 @@
         <v>4.9384341871337332E-3</v>
       </c>
       <c r="E82" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>8.4126226377823148</v>
       </c>
       <c r="F82" s="5">
@@ -12651,7 +12982,7 @@
         <v>0.81360703233028242</v>
       </c>
       <c r="K82" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>79.091492724040307</v>
       </c>
       <c r="L82" s="5">
@@ -12670,23 +13001,27 @@
         <v>2.5498781852900505</v>
       </c>
       <c r="Q82" s="5">
+        <f t="shared" si="6"/>
         <v>0.17531441364324751</v>
       </c>
       <c r="R82" s="5">
-        <v>0</v>
+        <v>0.17531441364324751</v>
       </c>
       <c r="S82" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T82" s="5">
+        <f t="shared" si="7"/>
         <v>0.76792651609929541</v>
       </c>
-      <c r="T82" s="5">
+      <c r="U82" s="5">
         <v>0.74282280898136566</v>
       </c>
-      <c r="U82" s="5">
+      <c r="V82" s="5">
         <v>2.5103707117929808E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>98</v>
       </c>
@@ -12700,7 +13035,7 @@
         <v>0.59556509661733681</v>
       </c>
       <c r="E83" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.820361339542536</v>
       </c>
       <c r="F83" s="5">
@@ -12719,7 +13054,7 @@
         <v>3.5797293756708557</v>
       </c>
       <c r="K83" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>84.156531636226362</v>
       </c>
       <c r="L83" s="5">
@@ -12738,23 +13073,27 @@
         <v>1.4518660006705038</v>
       </c>
       <c r="Q83" s="5">
+        <f t="shared" si="6"/>
+        <v>0.13691799288364506</v>
+      </c>
+      <c r="R83" s="5">
         <v>4.8738297878334558E-2</v>
       </c>
-      <c r="R83" s="5">
+      <c r="S83" s="5">
         <v>8.8179695005310504E-2</v>
       </c>
-      <c r="S83" s="5">
-        <f t="shared" si="5"/>
+      <c r="T83" s="5">
+        <f t="shared" si="7"/>
         <v>0.25876373757948146</v>
       </c>
-      <c r="T83" s="5">
+      <c r="U83" s="5">
         <v>0.24101510887234229</v>
       </c>
-      <c r="U83" s="5">
+      <c r="V83" s="5">
         <v>1.7748628707139176E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>99</v>
       </c>
@@ -12768,7 +13107,7 @@
         <v>6.2330150340322618E-2</v>
       </c>
       <c r="E84" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>6.1924191361149568</v>
       </c>
       <c r="F84" s="5">
@@ -12787,7 +13126,7 @@
         <v>1.4738641549603417</v>
       </c>
       <c r="K84" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>76.185654959799763</v>
       </c>
       <c r="L84" s="5">
@@ -12806,23 +13145,27 @@
         <v>2.5672975923217924</v>
       </c>
       <c r="Q84" s="5">
+        <f t="shared" si="6"/>
+        <v>1.9967870162502832</v>
+      </c>
+      <c r="R84" s="5">
         <v>1.8432922460208974</v>
       </c>
-      <c r="R84" s="5">
+      <c r="S84" s="5">
         <v>0.15349477022938579</v>
       </c>
-      <c r="S84" s="5">
-        <f t="shared" si="5"/>
+      <c r="T84" s="5">
+        <f t="shared" si="7"/>
         <v>2.4723389632815795</v>
       </c>
-      <c r="T84" s="5">
+      <c r="U84" s="5">
         <v>1.9741855617355748</v>
       </c>
-      <c r="U84" s="5">
+      <c r="V84" s="5">
         <v>0.49815340154600457</v>
       </c>
     </row>
-    <row r="85" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>100</v>
       </c>
@@ -12836,7 +13179,7 @@
         <v>0</v>
       </c>
       <c r="E85" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.1303994949950402</v>
       </c>
       <c r="F85" s="5">
@@ -12855,7 +13198,7 @@
         <v>0.12480836865362072</v>
       </c>
       <c r="K85" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>81.776896023085953</v>
       </c>
       <c r="L85" s="5">
@@ -12874,23 +13217,27 @@
         <v>2.5531607899720443</v>
       </c>
       <c r="Q85" s="5">
+        <f t="shared" si="6"/>
         <v>0.13310487870863016</v>
       </c>
       <c r="R85" s="5">
-        <v>0</v>
+        <v>0.13310487870863016</v>
       </c>
       <c r="S85" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T85" s="5">
+        <f t="shared" si="7"/>
         <v>2.0160519433673012</v>
       </c>
-      <c r="T85" s="5">
+      <c r="U85" s="5">
         <v>1.884029218144107</v>
       </c>
-      <c r="U85" s="5">
+      <c r="V85" s="5">
         <v>0.13202272522319414</v>
       </c>
     </row>
-    <row r="86" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>101</v>
       </c>
@@ -12904,7 +13251,7 @@
         <v>0</v>
       </c>
       <c r="E86" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>28.833856528310665</v>
       </c>
       <c r="F86" s="5">
@@ -12923,7 +13270,7 @@
         <v>0.39530287175909778</v>
       </c>
       <c r="K86" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>61.132426462039291</v>
       </c>
       <c r="L86" s="5">
@@ -12942,23 +13289,27 @@
         <v>2.1741657946750377</v>
       </c>
       <c r="Q86" s="5">
+        <f t="shared" si="6"/>
         <v>4.0576677130566212</v>
       </c>
       <c r="R86" s="5">
-        <v>0</v>
+        <v>4.0576677130566212</v>
       </c>
       <c r="S86" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T86" s="5">
+        <f t="shared" si="7"/>
         <v>1.6625973723985581</v>
       </c>
-      <c r="T86" s="5">
+      <c r="U86" s="5">
         <v>1.6625973723985581</v>
       </c>
-      <c r="U86" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V86" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>102</v>
       </c>
@@ -12972,7 +13323,7 @@
         <v>0</v>
       </c>
       <c r="E87" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>13.456147376852222</v>
       </c>
       <c r="F87" s="5">
@@ -12991,7 +13342,7 @@
         <v>0.12014417300760913</v>
       </c>
       <c r="K87" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>57.028434120945136</v>
       </c>
       <c r="L87" s="5">
@@ -13010,23 +13361,27 @@
         <v>0.88105726872246704</v>
       </c>
       <c r="Q87" s="5">
+        <f t="shared" si="6"/>
         <v>25.951141369643572</v>
       </c>
       <c r="R87" s="5">
-        <v>0</v>
+        <v>25.951141369643572</v>
       </c>
       <c r="S87" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T87" s="5">
+        <f t="shared" si="7"/>
         <v>0.28033640368442131</v>
       </c>
-      <c r="T87" s="5">
+      <c r="U87" s="5">
         <v>0.28033640368442131</v>
       </c>
-      <c r="U87" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V87" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>103</v>
       </c>
@@ -13040,7 +13395,7 @@
         <v>0</v>
       </c>
       <c r="E88" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>17.885996409335728</v>
       </c>
       <c r="F88" s="5">
@@ -13059,7 +13414,7 @@
         <v>0</v>
       </c>
       <c r="K88" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>79.555655296229801</v>
       </c>
       <c r="L88" s="5">
@@ -13078,23 +13433,27 @@
         <v>0.56104129263913827</v>
       </c>
       <c r="Q88" s="5">
+        <f t="shared" si="6"/>
         <v>0.33662477558348292</v>
       </c>
       <c r="R88" s="5">
-        <v>0</v>
+        <v>0.33662477558348292</v>
       </c>
       <c r="S88" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T88" s="5">
+        <f t="shared" si="7"/>
         <v>0.20197486535008977</v>
       </c>
-      <c r="T88" s="5">
+      <c r="U88" s="5">
         <v>0.13464991023339318</v>
       </c>
-      <c r="U88" s="5">
+      <c r="V88" s="5">
         <v>6.7324955116696589E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>104</v>
       </c>
@@ -13108,7 +13467,7 @@
         <v>0</v>
       </c>
       <c r="E89" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>16.230461650308978</v>
       </c>
       <c r="F89" s="5">
@@ -13127,7 +13486,7 @@
         <v>0.32715376226826609</v>
       </c>
       <c r="K89" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>60.814249363867681</v>
       </c>
       <c r="L89" s="5">
@@ -13146,23 +13505,27 @@
         <v>0.96328607778989461</v>
       </c>
       <c r="Q89" s="5">
+        <f t="shared" si="6"/>
         <v>19.683751363140676</v>
       </c>
       <c r="R89" s="5">
-        <v>0</v>
+        <v>19.683751363140676</v>
       </c>
       <c r="S89" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T89" s="5">
+        <f t="shared" si="7"/>
         <v>0.29080334423845872</v>
       </c>
-      <c r="T89" s="5">
+      <c r="U89" s="5">
         <v>0.29080334423845872</v>
       </c>
-      <c r="U89" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V89" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>105</v>
       </c>
@@ -13176,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="E90" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>20.449670882331191</v>
       </c>
       <c r="F90" s="5">
@@ -13195,7 +13558,7 @@
         <v>0.33281562014643884</v>
       </c>
       <c r="K90" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>60.239627246505435</v>
       </c>
       <c r="L90" s="5">
@@ -13214,23 +13577,27 @@
         <v>2.1152281635973673</v>
       </c>
       <c r="Q90" s="5">
+        <f t="shared" si="6"/>
         <v>10.420826861918497</v>
       </c>
       <c r="R90" s="5">
-        <v>0</v>
+        <v>10.420826861918497</v>
       </c>
       <c r="S90" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T90" s="5">
+        <f t="shared" si="7"/>
         <v>3.8236816803490865</v>
       </c>
-      <c r="T90" s="5">
+      <c r="U90" s="5">
         <v>3.6239923082612231</v>
       </c>
-      <c r="U90" s="5">
+      <c r="V90" s="5">
         <v>0.19968937208786333</v>
       </c>
     </row>
-    <row r="91" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>106</v>
       </c>
@@ -13244,7 +13611,7 @@
         <v>0</v>
       </c>
       <c r="E91" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10.74104912572856</v>
       </c>
       <c r="F91" s="5">
@@ -13263,7 +13630,7 @@
         <v>3.5803497085761866</v>
       </c>
       <c r="K91" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>73.522064945878441</v>
       </c>
       <c r="L91" s="5">
@@ -13282,23 +13649,27 @@
         <v>3.0807660283097418</v>
       </c>
       <c r="Q91" s="5">
+        <f t="shared" si="6"/>
         <v>4.4962531223980013</v>
       </c>
       <c r="R91" s="5">
-        <v>0</v>
+        <v>4.4962531223980013</v>
       </c>
       <c r="S91" s="5">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T91" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U91" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="92" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V91" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>107</v>
       </c>
@@ -13312,7 +13683,7 @@
         <v>0</v>
       </c>
       <c r="E92" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>61.242236024844722</v>
       </c>
       <c r="F92" s="5">
@@ -13331,7 +13702,7 @@
         <v>0.93167701863354035</v>
       </c>
       <c r="K92" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>33.850931677018636</v>
       </c>
       <c r="L92" s="5">
@@ -13350,23 +13721,27 @@
         <v>0.55900621118012428</v>
       </c>
       <c r="Q92" s="5">
+        <f t="shared" si="6"/>
         <v>1.9875776397515528</v>
       </c>
       <c r="R92" s="5">
-        <v>0</v>
+        <v>1.9875776397515528</v>
       </c>
       <c r="S92" s="5">
-        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T92" s="5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U92" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="93" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V92" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>108</v>
       </c>
@@ -13380,7 +13755,7 @@
         <v>0</v>
       </c>
       <c r="E93" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>15.885264814220072</v>
       </c>
       <c r="F93" s="5">
@@ -13399,7 +13774,7 @@
         <v>0.20992082217194488</v>
       </c>
       <c r="K93" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>75.91705795070628</v>
       </c>
       <c r="L93" s="5">
@@ -13418,23 +13793,27 @@
         <v>0.54651181567157614</v>
       </c>
       <c r="Q93" s="5">
+        <f t="shared" si="6"/>
         <v>0.56678621986425126</v>
       </c>
       <c r="R93" s="5">
-        <v>0</v>
+        <v>0.56678621986425126</v>
       </c>
       <c r="S93" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T93" s="5">
+        <f t="shared" si="7"/>
         <v>1.5356515529655355</v>
       </c>
-      <c r="T93" s="5">
+      <c r="U93" s="5">
         <v>1.3992927283068362</v>
       </c>
-      <c r="U93" s="5">
+      <c r="V93" s="5">
         <v>0.13635882465869922</v>
       </c>
     </row>
-    <row r="94" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>109</v>
       </c>
@@ -13448,7 +13827,7 @@
         <v>0</v>
       </c>
       <c r="E94" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>20.440616200099385</v>
       </c>
       <c r="F94" s="5">
@@ -13467,7 +13846,7 @@
         <v>2.4846778201093257E-2</v>
       </c>
       <c r="K94" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>77.836673844624812</v>
       </c>
       <c r="L94" s="5">
@@ -13486,33 +13865,37 @@
         <v>0.37270167301639889</v>
       </c>
       <c r="Q94" s="5">
+        <f t="shared" si="6"/>
         <v>0.25675004141129698</v>
       </c>
       <c r="R94" s="5">
-        <v>0</v>
+        <v>0.25675004141129698</v>
       </c>
       <c r="S94" s="5">
-        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T94" s="5">
+        <f t="shared" si="7"/>
         <v>0.14908066920655955</v>
       </c>
-      <c r="T94" s="5">
+      <c r="U94" s="5">
         <v>0.10766937220473745</v>
       </c>
-      <c r="U94" s="5">
+      <c r="V94" s="5">
         <v>4.1411297001822098E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="S96" s="5"/>
-    </row>
-    <row r="97" spans="19:19" x14ac:dyDescent="0.3">
-      <c r="S97" s="5"/>
-    </row>
-    <row r="98" spans="19:19" x14ac:dyDescent="0.3">
-      <c r="S98" s="5"/>
-    </row>
-    <row r="99" spans="19:19" x14ac:dyDescent="0.3">
-      <c r="S99" s="5"/>
+    <row r="96" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="T96" s="5"/>
+    </row>
+    <row r="97" spans="20:20" x14ac:dyDescent="0.3">
+      <c r="T97" s="5"/>
+    </row>
+    <row r="98" spans="20:20" x14ac:dyDescent="0.3">
+      <c r="T98" s="5"/>
+    </row>
+    <row r="99" spans="20:20" x14ac:dyDescent="0.3">
+      <c r="T99" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Made Edits, Fixed trends function, working on landcover model function. plots
</commit_message>
<xml_diff>
--- a/data_cache/streams_2019lulc.xlsx
+++ b/data_cache/streams_2019lulc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/530e20b7f6c3b906/Documents/KC-Streams-Analysis/data_cache/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{E3052FD2-981D-4E2C-8B81-FC6F18F19128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7716A1CF-BC1C-470A-8D80-971234F3CCB4}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="8_{E3052FD2-981D-4E2C-8B81-FC6F18F19128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C04F9D66-F4B5-4C77-AEE6-16CBB54E5035}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14856" activeTab="1" xr2:uid="{B79C8CA6-09B2-4EB5-862A-BB01EB8BD711}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="13545" activeTab="1" xr2:uid="{B79C8CA6-09B2-4EB5-862A-BB01EB8BD711}"/>
   </bookViews>
   <sheets>
     <sheet name="LULC - sq m" sheetId="1" r:id="rId1"/>
@@ -573,9 +573,6 @@
     <t>Stream</t>
   </si>
   <si>
-    <t>Urban, Total</t>
-  </si>
-  <si>
     <t>Forest, Total</t>
   </si>
   <si>
@@ -583,6 +580,9 @@
   </si>
   <si>
     <t>Agriculture, Total</t>
+  </si>
+  <si>
+    <t>Developed, All Intensities</t>
   </si>
 </sst>
 </file>
@@ -992,30 +992,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4283B9C-F0A7-40D0-A9F5-705AEC2E6A72}">
   <dimension ref="A1:T95"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.33203125" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
-    <col min="15" max="15" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="11" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" s="7" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="6"/>
       <c r="B1" s="1"/>
       <c r="C1" s="4" t="s">
@@ -1073,7 +1073,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1199,7 +1199,7 @@
         <v>1230.4521</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1263,7 +1263,7 @@
         <v>1208.0546999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1327,7 +1327,7 @@
         <v>1198.0143</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>1191.3290999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1455,7 +1455,7 @@
         <v>1113.0029999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1519,7 +1519,7 @@
         <v>57.198599999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1583,7 +1583,7 @@
         <v>10.8531</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>80.406899999999993</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1711,7 +1711,7 @@
         <v>9.5103000000000009</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -1775,7 +1775,7 @@
         <v>30.5793</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -1839,7 +1839,7 @@
         <v>493.96319999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>33.426900000000003</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -1967,7 +1967,7 @@
         <v>15.426</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -2031,7 +2031,7 @@
         <v>36.586799999999997</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>31</v>
       </c>
@@ -2095,7 +2095,7 @@
         <v>16.642800000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -2159,7 +2159,7 @@
         <v>626.36310000000003</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>33</v>
       </c>
@@ -2223,7 +2223,7 @@
         <v>7.5941999999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>34</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>63.617400000000004</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -2351,7 +2351,7 @@
         <v>74.015100000000004</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>36</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>38.960999999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>123.5313</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>38</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>262.95929999999998</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>39</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>1.6820999999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>40</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>144.94409999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>41</v>
       </c>
@@ -2735,7 +2735,7 @@
         <v>10.461600000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>42</v>
       </c>
@@ -2799,7 +2799,7 @@
         <v>1113.2424000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>43</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>419.54489999999998</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>44</v>
       </c>
@@ -2927,7 +2927,7 @@
         <v>7.5941999999999998</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>45</v>
       </c>
@@ -2991,7 +2991,7 @@
         <v>124.42140000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>46</v>
       </c>
@@ -3055,7 +3055,7 @@
         <v>33.795000000000002</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>47</v>
       </c>
@@ -3119,7 +3119,7 @@
         <v>831.85919999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>48</v>
       </c>
@@ -3183,7 +3183,7 @@
         <v>173.89080000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>49</v>
       </c>
@@ -3247,7 +3247,7 @@
         <v>20.398499999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>50</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>446.77530000000002</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>51</v>
       </c>
@@ -3375,7 +3375,7 @@
         <v>6.6914999999999996</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>52</v>
       </c>
@@ -3439,7 +3439,7 @@
         <v>0.62729999999999997</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>53</v>
       </c>
@@ -3503,7 +3503,7 @@
         <v>4.6656000000000004</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>54</v>
       </c>
@@ -3567,7 +3567,7 @@
         <v>1.3031999999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>55</v>
       </c>
@@ -3631,7 +3631,7 @@
         <v>105.8355</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>56</v>
       </c>
@@ -3695,7 +3695,7 @@
         <v>10.212300000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>57</v>
       </c>
@@ -3759,7 +3759,7 @@
         <v>15.111000000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>58</v>
       </c>
@@ -3823,7 +3823,7 @@
         <v>4.7664</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>59</v>
       </c>
@@ -3887,7 +3887,7 @@
         <v>3.2570999999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>60</v>
       </c>
@@ -3951,7 +3951,7 @@
         <v>0.55259999999999998</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>61</v>
       </c>
@@ -4015,7 +4015,7 @@
         <v>10.7226</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>62</v>
       </c>
@@ -4079,7 +4079,7 @@
         <v>18.845099999999999</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>63</v>
       </c>
@@ -4143,7 +4143,7 @@
         <v>710.06849999999997</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>64</v>
       </c>
@@ -4207,7 +4207,7 @@
         <v>33.0471</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>65</v>
       </c>
@@ -4271,7 +4271,7 @@
         <v>7.3259999999999996</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>66</v>
       </c>
@@ -4335,7 +4335,7 @@
         <v>55.584899999999998</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>67</v>
       </c>
@@ -4399,7 +4399,7 @@
         <v>41.693399999999997</v>
       </c>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>68</v>
       </c>
@@ -4463,7 +4463,7 @@
         <v>17.979299999999999</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>69</v>
       </c>
@@ -4527,7 +4527,7 @@
         <v>9.8036999999999992</v>
       </c>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>70</v>
       </c>
@@ -4591,7 +4591,7 @@
         <v>7.1288999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>71</v>
       </c>
@@ -4655,7 +4655,7 @@
         <v>84.224699999999999</v>
       </c>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>72</v>
       </c>
@@ -4719,7 +4719,7 @@
         <v>53.442900000000002</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>73</v>
       </c>
@@ -4783,7 +4783,7 @@
         <v>42.198300000000003</v>
       </c>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>74</v>
       </c>
@@ -4847,7 +4847,7 @@
         <v>21.307500000000001</v>
       </c>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>75</v>
       </c>
@@ -4911,7 +4911,7 @@
         <v>66.509100000000004</v>
       </c>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>76</v>
       </c>
@@ -4975,7 +4975,7 @@
         <v>6.0471000000000004</v>
       </c>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>77</v>
       </c>
@@ -5039,7 +5039,7 @@
         <v>6.0389999999999997</v>
       </c>
     </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>78</v>
       </c>
@@ -5103,7 +5103,7 @@
         <v>9.6173999999999999</v>
       </c>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>79</v>
       </c>
@@ -5167,7 +5167,7 @@
         <v>43.065899999999999</v>
       </c>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>80</v>
       </c>
@@ -5231,7 +5231,7 @@
         <v>21.096900000000002</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>81</v>
       </c>
@@ -5295,7 +5295,7 @@
         <v>5.6780999999999997</v>
       </c>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>82</v>
       </c>
@@ -5359,7 +5359,7 @@
         <v>35.454599999999999</v>
       </c>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>83</v>
       </c>
@@ -5423,7 +5423,7 @@
         <v>6.5646000000000004</v>
       </c>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>84</v>
       </c>
@@ -5487,7 +5487,7 @@
         <v>4.3415999999999997</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>85</v>
       </c>
@@ -5551,7 +5551,7 @@
         <v>4.5035999999999996</v>
       </c>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>86</v>
       </c>
@@ -5615,7 +5615,7 @@
         <v>1.6541999999999999</v>
       </c>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>87</v>
       </c>
@@ -5679,7 +5679,7 @@
         <v>17.742599999999999</v>
       </c>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>88</v>
       </c>
@@ -5743,7 +5743,7 @@
         <v>8.6021999999999998</v>
       </c>
     </row>
-    <row r="75" spans="1:20" ht="27" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:20" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>89</v>
       </c>
@@ -5807,7 +5807,7 @@
         <v>442.74869999999999</v>
       </c>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:20" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>90</v>
       </c>
@@ -5871,7 +5871,7 @@
         <v>27.520199999999999</v>
       </c>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:20" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>91</v>
       </c>
@@ -5935,7 +5935,7 @@
         <v>27.1557</v>
       </c>
     </row>
-    <row r="78" spans="1:20" ht="27" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:20" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>92</v>
       </c>
@@ -5999,7 +5999,7 @@
         <v>266.89589999999998</v>
       </c>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>93</v>
       </c>
@@ -6063,7 +6063,7 @@
         <v>52.862400000000001</v>
       </c>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>94</v>
       </c>
@@ -6127,7 +6127,7 @@
         <v>83.645099999999999</v>
       </c>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>95</v>
       </c>
@@ -6191,7 +6191,7 @@
         <v>14.453099999999999</v>
       </c>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>96</v>
       </c>
@@ -6255,7 +6255,7 @@
         <v>24.452100000000002</v>
       </c>
     </row>
-    <row r="83" spans="1:20" ht="27" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:20" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>97</v>
       </c>
@@ -6319,7 +6319,7 @@
         <v>218.69280000000001</v>
       </c>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>98</v>
       </c>
@@ -6383,7 +6383,7 @@
         <v>638.92259999999999</v>
       </c>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>99</v>
       </c>
@@ -6447,7 +6447,7 @@
         <v>1660.5126</v>
       </c>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>100</v>
       </c>
@@ -6511,7 +6511,7 @@
         <v>249.5025</v>
       </c>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>101</v>
       </c>
@@ -6575,7 +6575,7 @@
         <v>7.7408999999999999</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>102</v>
       </c>
@@ -6639,7 +6639,7 @@
         <v>2.2473000000000001</v>
       </c>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>103</v>
       </c>
@@ -6703,7 +6703,7 @@
         <v>4.0103999999999997</v>
       </c>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>104</v>
       </c>
@@ -6767,7 +6767,7 @@
         <v>4.9518000000000004</v>
       </c>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>105</v>
       </c>
@@ -6831,7 +6831,7 @@
         <v>12.168900000000001</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>106</v>
       </c>
@@ -6895,7 +6895,7 @@
         <v>1.0809</v>
       </c>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>107</v>
       </c>
@@ -6959,7 +6959,7 @@
         <v>1.4490000000000001</v>
       </c>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>108</v>
       </c>
@@ -7023,7 +7023,7 @@
         <v>501.61770000000001</v>
       </c>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>109</v>
       </c>
@@ -7095,33 +7095,33 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DA31AB4-F286-4205-A346-ED4D5FE79DEC}">
   <dimension ref="A1:V100"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.44140625" customWidth="1"/>
-    <col min="10" max="10" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.44140625" customWidth="1"/>
-    <col min="12" max="12" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" customWidth="1"/>
+    <col min="12" max="12" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.109375" customWidth="1"/>
-    <col min="18" max="18" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.109375" customWidth="1"/>
-    <col min="21" max="21" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.140625" customWidth="1"/>
+    <col min="18" max="18" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.140625" customWidth="1"/>
+    <col min="21" max="21" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>15</v>
       </c>
@@ -7135,7 +7135,7 @@
         <v>1</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>2</v>
@@ -7153,7 +7153,7 @@
         <v>6</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L1" s="4" t="s">
         <v>7</v>
@@ -7171,7 +7171,7 @@
         <v>11</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="R1" s="4" t="s">
         <v>12</v>
@@ -7180,7 +7180,7 @@
         <v>13</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>14</v>
@@ -7189,7 +7189,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -7203,8 +7203,8 @@
         <v>0</v>
       </c>
       <c r="E2" s="5">
-        <f>SUM(F2:I2)</f>
-        <v>28.1395350538229</v>
+        <f>SUM(G2:I2)</f>
+        <v>21.20191432076064</v>
       </c>
       <c r="F2" s="5">
         <v>6.9376207330622623</v>
@@ -7261,7 +7261,7 @@
         <v>0.54301991926382176</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -7275,8 +7275,8 @@
         <v>0</v>
       </c>
       <c r="E3" s="5">
-        <f t="shared" ref="E3:E66" si="0">SUM(F3:I3)</f>
-        <v>27.054354409614071</v>
+        <f t="shared" ref="E3:E66" si="0">SUM(G3:I3)</f>
+        <v>20.05881025089344</v>
       </c>
       <c r="F3" s="5">
         <v>6.9955441587206275</v>
@@ -7333,7 +7333,7 @@
         <v>0.54817054227759721</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -7348,7 +7348,7 @@
       </c>
       <c r="E4" s="5">
         <f t="shared" si="0"/>
-        <v>26.502279647246283</v>
+        <v>19.509934063391398</v>
       </c>
       <c r="F4" s="5">
         <v>6.9923455838548838</v>
@@ -7405,7 +7405,7 @@
         <v>0.54983483920016651</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="E5" s="5">
         <f t="shared" si="0"/>
-        <v>26.123159419173092</v>
+        <v>19.145440164266951</v>
       </c>
       <c r="F5" s="5">
         <v>6.9777192549061384</v>
@@ -7477,7 +7477,7 @@
         <v>0.55065388732634835</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -7492,7 +7492,7 @@
       </c>
       <c r="E6" s="5">
         <f t="shared" si="0"/>
-        <v>21.504119934986697</v>
+        <v>14.59306039606362</v>
       </c>
       <c r="F6" s="5">
         <v>6.9110595389230758</v>
@@ -7549,7 +7549,7 @@
         <v>0.50959431376195752</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -7564,7 +7564,7 @@
       </c>
       <c r="E7" s="5">
         <f t="shared" si="0"/>
-        <v>91.249960663372889</v>
+        <v>83.741385278660672</v>
       </c>
       <c r="F7" s="5">
         <v>7.5085753847122128</v>
@@ -7621,7 +7621,7 @@
         <v>1.464895993957894</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -7636,7 +7636,7 @@
       </c>
       <c r="E8" s="5">
         <f t="shared" si="0"/>
-        <v>26.735218508997434</v>
+        <v>15.457334770710673</v>
       </c>
       <c r="F8" s="5">
         <v>11.277883738286757</v>
@@ -7693,7 +7693,7 @@
         <v>0.33170246289078698</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -7708,7 +7708,7 @@
       </c>
       <c r="E9" s="5">
         <f t="shared" si="0"/>
-        <v>25.977994425851513</v>
+        <v>15.962436059591901</v>
       </c>
       <c r="F9" s="5">
         <v>10.015558366259611</v>
@@ -7765,7 +7765,7 @@
         <v>1.5659103882875725</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -7780,7 +7780,7 @@
       </c>
       <c r="E10" s="5">
         <f t="shared" si="0"/>
-        <v>89.826819343238384</v>
+        <v>79.805053468344852</v>
       </c>
       <c r="F10" s="5">
         <v>10.021765874893536</v>
@@ -7837,7 +7837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -7852,7 +7852,7 @@
       </c>
       <c r="E11" s="5">
         <f t="shared" si="0"/>
-        <v>97.633693380816439</v>
+        <v>92.085822762456971</v>
       </c>
       <c r="F11" s="5">
         <v>5.5478706183594788</v>
@@ -7909,7 +7909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -7923,8 +7923,8 @@
         <v>0</v>
       </c>
       <c r="E12" s="5">
-        <f t="shared" si="0"/>
-        <v>14.584730198524911</v>
+        <f>SUM(G12:I12)</f>
+        <v>8.634995481444772</v>
       </c>
       <c r="F12" s="5">
         <v>5.9497347170801387</v>
@@ -7981,7 +7981,7 @@
         <v>0.13774305454333441</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -7996,7 +7996,7 @@
       </c>
       <c r="E13" s="5">
         <f t="shared" si="0"/>
-        <v>51.877978514310328</v>
+        <v>36.2698904175978</v>
       </c>
       <c r="F13" s="5">
         <v>15.608088096712528</v>
@@ -8053,7 +8053,7 @@
         <v>0.51425648205487196</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -8068,7 +8068,7 @@
       </c>
       <c r="E14" s="5">
         <f t="shared" si="0"/>
-        <v>56.913652275379235</v>
+        <v>44.189031505250881</v>
       </c>
       <c r="F14" s="5">
         <v>12.724620770128356</v>
@@ -8125,7 +8125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -8140,7 +8140,7 @@
       </c>
       <c r="E15" s="5">
         <f t="shared" si="0"/>
-        <v>87.34871593033553</v>
+        <v>77.10075765030011</v>
       </c>
       <c r="F15" s="5">
         <v>10.247958280035423</v>
@@ -8197,7 +8197,7 @@
         <v>0.63711502509101636</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -8212,7 +8212,7 @@
       </c>
       <c r="E16" s="5">
         <f t="shared" si="0"/>
-        <v>91.396279472204185</v>
+        <v>84.696084793424177</v>
       </c>
       <c r="F16" s="5">
         <v>6.7001946787800124</v>
@@ -8269,7 +8269,7 @@
         <v>0.1081548777849881</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -8284,7 +8284,7 @@
       </c>
       <c r="E17" s="5">
         <f t="shared" si="0"/>
-        <v>57.931860928589188</v>
+        <v>43.022649322733095</v>
       </c>
       <c r="F17" s="5">
         <v>14.909211605856093</v>
@@ -8341,7 +8341,7 @@
         <v>0.83711827851928067</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>33</v>
       </c>
@@ -8356,7 +8356,7 @@
       </c>
       <c r="E18" s="5">
         <f t="shared" si="0"/>
-        <v>91.064233230623373</v>
+        <v>79.947854941929364</v>
       </c>
       <c r="F18" s="5">
         <v>11.116378288694003</v>
@@ -8413,7 +8413,7 @@
         <v>0.35553448684522398</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>34</v>
       </c>
@@ -8428,7 +8428,7 @@
       </c>
       <c r="E19" s="5">
         <f t="shared" si="0"/>
-        <v>89.484480660951263</v>
+        <v>77.344877344877347</v>
       </c>
       <c r="F19" s="5">
         <v>12.139603316073904</v>
@@ -8485,7 +8485,7 @@
         <v>0.41592394533571003</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -8500,7 +8500,7 @@
       </c>
       <c r="E20" s="5">
         <f t="shared" si="0"/>
-        <v>87.459721056919477</v>
+        <v>73.496759445032154</v>
       </c>
       <c r="F20" s="5">
         <v>13.962961611887303</v>
@@ -8557,7 +8557,7 @@
         <v>1.1539537202543806</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -8572,7 +8572,7 @@
       </c>
       <c r="E21" s="5">
         <f t="shared" si="0"/>
-        <v>69.029799029799022</v>
+        <v>43.028413028413027</v>
       </c>
       <c r="F21" s="5">
         <v>26.001386001386003</v>
@@ -8629,7 +8629,7 @@
         <v>0.12936012936012936</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>37</v>
       </c>
@@ -8644,7 +8644,7 @@
       </c>
       <c r="E22" s="5">
         <f t="shared" si="0"/>
-        <v>56.035029178839693</v>
+        <v>32.931653759006828</v>
       </c>
       <c r="F22" s="5">
         <v>23.103375419832869</v>
@@ -8701,7 +8701,7 @@
         <v>1.3842645548132335</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>38</v>
       </c>
@@ -8716,7 +8716,7 @@
       </c>
       <c r="E23" s="5">
         <f t="shared" si="0"/>
-        <v>36.844104772107315</v>
+        <v>26.323084979310483</v>
       </c>
       <c r="F23" s="5">
         <v>10.521019792796832</v>
@@ -8773,7 +8773,7 @@
         <v>0.66603462969364458</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>39</v>
       </c>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="E24" s="5">
         <f t="shared" si="0"/>
-        <v>99.197431781701454</v>
+        <v>76.565008025682189</v>
       </c>
       <c r="F24" s="5">
         <v>22.632423756019264</v>
@@ -8845,7 +8845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>40</v>
       </c>
@@ -8860,7 +8860,7 @@
       </c>
       <c r="E25" s="5">
         <f t="shared" si="0"/>
-        <v>21.190445144024491</v>
+        <v>12.550838564660443</v>
       </c>
       <c r="F25" s="5">
         <v>8.6396065793640435</v>
@@ -8917,7 +8917,7 @@
         <v>0.13660438748455439</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>41</v>
       </c>
@@ -8932,7 +8932,7 @@
       </c>
       <c r="E26" s="5">
         <f t="shared" si="0"/>
-        <v>46.83413626978664</v>
+        <v>38.205437026841025</v>
       </c>
       <c r="F26" s="5">
         <v>8.6286992429456291</v>
@@ -8989,7 +8989,7 @@
         <v>0.27529249827942187</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>42</v>
       </c>
@@ -9004,7 +9004,7 @@
       </c>
       <c r="E27" s="5">
         <f t="shared" si="0"/>
-        <v>21.519868449135608</v>
+        <v>14.609082442422245</v>
       </c>
       <c r="F27" s="5">
         <v>6.9107860067133622</v>
@@ -9061,7 +9061,7 @@
         <v>0.50948472677648649</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>43</v>
       </c>
@@ -9076,7 +9076,7 @@
       </c>
       <c r="E28" s="5">
         <f t="shared" si="0"/>
-        <v>45.622220649089044</v>
+        <v>31.146964246258264</v>
       </c>
       <c r="F28" s="5">
         <v>14.475256402830784</v>
@@ -9133,7 +9133,7 @@
         <v>0.89582783630548246</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>44</v>
       </c>
@@ -9148,7 +9148,7 @@
       </c>
       <c r="E29" s="5">
         <f t="shared" si="0"/>
-        <v>91.064233230623373</v>
+        <v>79.947854941929364</v>
       </c>
       <c r="F29" s="5">
         <v>11.116378288694003</v>
@@ -9205,7 +9205,7 @@
         <v>0.35553448684522398</v>
       </c>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>45</v>
       </c>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="E30" s="5">
         <f t="shared" si="0"/>
-        <v>56.315553433734067</v>
+        <v>33.33695007450487</v>
       </c>
       <c r="F30" s="5">
         <v>22.978603359229201</v>
@@ -9277,7 +9277,7 @@
         <v>1.393168699275205</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>46</v>
       </c>
@@ -9292,7 +9292,7 @@
       </c>
       <c r="E31" s="5">
         <f t="shared" si="0"/>
-        <v>81.294274300932088</v>
+        <v>69.645805592543269</v>
       </c>
       <c r="F31" s="5">
         <v>11.648468708388815</v>
@@ -9349,7 +9349,7 @@
         <v>4.2583222370173104</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>47</v>
       </c>
@@ -9364,7 +9364,7 @@
       </c>
       <c r="E32" s="5">
         <f t="shared" si="0"/>
-        <v>6.5281600540091409</v>
+        <v>2.9568705857914415</v>
       </c>
       <c r="F32" s="5">
         <v>3.5712894682176985</v>
@@ -9421,7 +9421,7 @@
         <v>0.24884018833956517</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>48</v>
       </c>
@@ -9436,7 +9436,7 @@
       </c>
       <c r="E33" s="5">
         <f t="shared" si="0"/>
-        <v>59.274268678964042</v>
+        <v>38.981533238101157</v>
       </c>
       <c r="F33" s="5">
         <v>20.292735440862884</v>
@@ -9493,7 +9493,7 @@
         <v>0.41146512638966526</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>49</v>
       </c>
@@ -9508,7 +9508,7 @@
       </c>
       <c r="E34" s="5">
         <f t="shared" si="0"/>
-        <v>93.187734392234731</v>
+        <v>84.138539598499889</v>
       </c>
       <c r="F34" s="5">
         <v>9.0491947937348343</v>
@@ -9565,7 +9565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>50</v>
       </c>
@@ -9580,7 +9580,7 @@
       </c>
       <c r="E35" s="5">
         <f t="shared" si="0"/>
-        <v>8.9771301143997881</v>
+        <v>4.0768144523656522</v>
       </c>
       <c r="F35" s="5">
         <v>4.9003156620341368</v>
@@ -9637,7 +9637,7 @@
         <v>0.14584512617416406</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>51</v>
       </c>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="E36" s="5">
         <f t="shared" si="0"/>
-        <v>93.006052454606589</v>
+        <v>82.273032952252862</v>
       </c>
       <c r="F36" s="5">
         <v>10.733019502353732</v>
@@ -9709,7 +9709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>52</v>
       </c>
@@ -9724,7 +9724,7 @@
       </c>
       <c r="E37" s="5">
         <f t="shared" si="0"/>
-        <v>66.140602582496413</v>
+        <v>57.675753228120513</v>
       </c>
       <c r="F37" s="5">
         <v>8.4648493543758967</v>
@@ -9781,7 +9781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>53</v>
       </c>
@@ -9796,7 +9796,7 @@
       </c>
       <c r="E38" s="5">
         <f t="shared" si="0"/>
-        <v>73.128858024691368</v>
+        <v>58.545524691358018</v>
       </c>
       <c r="F38" s="5">
         <v>14.583333333333334</v>
@@ -9853,7 +9853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>54</v>
       </c>
@@ -9868,7 +9868,7 @@
       </c>
       <c r="E39" s="5">
         <f t="shared" si="0"/>
-        <v>91.229281767955797</v>
+        <v>87.361878453038671</v>
       </c>
       <c r="F39" s="5">
         <v>3.867403314917127</v>
@@ -9925,7 +9925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>55</v>
       </c>
@@ -9940,7 +9940,7 @@
       </c>
       <c r="E40" s="5">
         <f t="shared" si="0"/>
-        <v>17.947191632297294</v>
+        <v>8.4238275436880823</v>
       </c>
       <c r="F40" s="5">
         <v>9.5233640886092097</v>
@@ -9997,7 +9997,7 @@
         <v>0.13606020664143884</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>56</v>
       </c>
@@ -10012,7 +10012,7 @@
       </c>
       <c r="E41" s="5">
         <f t="shared" si="0"/>
-        <v>45.606768308804085</v>
+        <v>37.225698422490524</v>
       </c>
       <c r="F41" s="5">
         <v>8.3810698863135631</v>
@@ -10069,7 +10069,7 @@
         <v>0.2820128668370494</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>57</v>
       </c>
@@ -10084,7 +10084,7 @@
       </c>
       <c r="E42" s="5">
         <f t="shared" si="0"/>
-        <v>74.556283502084568</v>
+        <v>54.359737939249555</v>
       </c>
       <c r="F42" s="5">
         <v>20.196545562835023</v>
@@ -10141,7 +10141,7 @@
         <v>0.47051816557474685</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>58</v>
       </c>
@@ -10156,7 +10156,7 @@
       </c>
       <c r="E43" s="5">
         <f t="shared" si="0"/>
-        <v>64.312688821752261</v>
+        <v>38.614048338368576</v>
       </c>
       <c r="F43" s="5">
         <v>25.698640483383684</v>
@@ -10213,7 +10213,7 @@
         <v>0.15105740181268881</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>59</v>
       </c>
@@ -10228,7 +10228,7 @@
       </c>
       <c r="E44" s="5">
         <f t="shared" si="0"/>
-        <v>70.212765957446805</v>
+        <v>41.862392926222704</v>
       </c>
       <c r="F44" s="5">
         <v>28.350373031224095</v>
@@ -10285,7 +10285,7 @@
         <v>5.5263885051119094E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>60</v>
       </c>
@@ -10300,7 +10300,7 @@
       </c>
       <c r="E45" s="5">
         <f t="shared" si="0"/>
-        <v>66.286644951140062</v>
+        <v>45.114006514657973</v>
       </c>
       <c r="F45" s="5">
         <v>21.172638436482085</v>
@@ -10357,7 +10357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>61</v>
       </c>
@@ -10372,7 +10372,7 @@
       </c>
       <c r="E46" s="5">
         <f t="shared" si="0"/>
-        <v>72.200772200772207</v>
+        <v>47.490347490347496</v>
       </c>
       <c r="F46" s="5">
         <v>24.710424710424711</v>
@@ -10429,7 +10429,7 @@
         <v>0.57075709249622297</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>62</v>
       </c>
@@ -10444,7 +10444,7 @@
       </c>
       <c r="E47" s="5">
         <f t="shared" si="0"/>
-        <v>19.146091026314533</v>
+        <v>8.5438655141124222</v>
       </c>
       <c r="F47" s="5">
         <v>10.602225512202111</v>
@@ -10501,7 +10501,7 @@
         <v>0.75934858398204308</v>
       </c>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>63</v>
       </c>
@@ -10516,7 +10516,7 @@
       </c>
       <c r="E48" s="5">
         <f t="shared" si="0"/>
-        <v>3.3114269961278384</v>
+        <v>0.94161337955422619</v>
       </c>
       <c r="F48" s="5">
         <v>2.3698136165736123</v>
@@ -10573,7 +10573,7 @@
         <v>6.6162630788438023E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>64</v>
       </c>
@@ -10588,7 +10588,7 @@
       </c>
       <c r="E49" s="5">
         <f t="shared" si="0"/>
-        <v>56.515700318636135</v>
+        <v>33.285220185734907</v>
       </c>
       <c r="F49" s="5">
         <v>23.230480132901224</v>
@@ -10645,7 +10645,7 @@
         <v>2.922192870176203</v>
       </c>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>65</v>
       </c>
@@ -10660,7 +10660,7 @@
       </c>
       <c r="E50" s="5">
         <f t="shared" si="0"/>
-        <v>73.476658476658471</v>
+        <v>64.103194103194099</v>
       </c>
       <c r="F50" s="5">
         <v>9.3734643734643743</v>
@@ -10717,7 +10717,7 @@
         <v>0.92137592137592139</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>66</v>
       </c>
@@ -10732,7 +10732,7 @@
       </c>
       <c r="E51" s="5">
         <f t="shared" si="0"/>
-        <v>90.877738378588447</v>
+        <v>79.321902171273138</v>
       </c>
       <c r="F51" s="5">
         <v>11.555836207315295</v>
@@ -10789,7 +10789,7 @@
         <v>5.6670066870678909E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>67</v>
       </c>
@@ -10804,7 +10804,7 @@
       </c>
       <c r="E52" s="5">
         <f t="shared" si="0"/>
-        <v>15.367180417044423</v>
+        <v>10.605275655139662</v>
       </c>
       <c r="F52" s="5">
         <v>4.7619047619047619</v>
@@ -10861,7 +10861,7 @@
         <v>0.6626948150066917</v>
       </c>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>68</v>
       </c>
@@ -10876,7 +10876,7 @@
       </c>
       <c r="E53" s="5">
         <f t="shared" si="0"/>
-        <v>57.4911147819993</v>
+        <v>34.039145016769289</v>
       </c>
       <c r="F53" s="5">
         <v>23.451969765230015</v>
@@ -10933,7 +10933,7 @@
         <v>8.0092105921810083E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>69</v>
       </c>
@@ -10948,7 +10948,7 @@
       </c>
       <c r="E54" s="5">
         <f t="shared" si="0"/>
-        <v>93.885981823189212</v>
+        <v>85.128063894244008</v>
       </c>
       <c r="F54" s="5">
         <v>8.7579179289451936</v>
@@ -11005,7 +11005,7 @@
         <v>6.4261452308822187E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>70</v>
       </c>
@@ -11020,7 +11020,7 @@
       </c>
       <c r="E55" s="5">
         <f t="shared" si="0"/>
-        <v>90.468375205150849</v>
+        <v>81.971973235702549</v>
       </c>
       <c r="F55" s="5">
         <v>8.4964019694483017</v>
@@ -11077,7 +11077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>71</v>
       </c>
@@ -11092,7 +11092,7 @@
       </c>
       <c r="E56" s="5">
         <f t="shared" si="0"/>
-        <v>55.282476518171038</v>
+        <v>31.254608208755862</v>
       </c>
       <c r="F56" s="5">
         <v>24.027868309415172</v>
@@ -11149,7 +11149,7 @@
         <v>0.65930778025923509</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>72</v>
       </c>
@@ -11164,7 +11164,7 @@
       </c>
       <c r="E57" s="5">
         <f t="shared" si="0"/>
-        <v>6.2292652531954662</v>
+        <v>2.0511611458210539</v>
       </c>
       <c r="F57" s="5">
         <v>4.1781041073744127</v>
@@ -11221,7 +11221,7 @@
         <v>6.2309492935450732E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>73</v>
       </c>
@@ -11236,7 +11236,7 @@
       </c>
       <c r="E58" s="5">
         <f t="shared" si="0"/>
-        <v>67.724529187194747</v>
+        <v>45.462494934630072</v>
       </c>
       <c r="F58" s="5">
         <v>22.262034252564678</v>
@@ -11293,7 +11293,7 @@
         <v>0.13863117708533282</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>74</v>
       </c>
@@ -11308,7 +11308,7 @@
       </c>
       <c r="E59" s="5">
         <f t="shared" si="0"/>
-        <v>87.488912354804654</v>
+        <v>75.417106652587108</v>
       </c>
       <c r="F59" s="5">
         <v>12.07180570221753</v>
@@ -11365,7 +11365,7 @@
         <v>0.21119324181626187</v>
       </c>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>75</v>
       </c>
@@ -11380,7 +11380,7 @@
       </c>
       <c r="E60" s="5">
         <f t="shared" si="0"/>
-        <v>88.101327487516755</v>
+        <v>74.298704989242083</v>
       </c>
       <c r="F60" s="5">
         <v>13.802622498274673</v>
@@ -11437,7 +11437,7 @@
         <v>1.083911825599805</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>76</v>
       </c>
@@ -11452,7 +11452,7 @@
       </c>
       <c r="E61" s="5">
         <f t="shared" si="0"/>
-        <v>27.608275040928714</v>
+        <v>16.966810537282331</v>
       </c>
       <c r="F61" s="5">
         <v>10.641464503646377</v>
@@ -11509,7 +11509,7 @@
         <v>0.52091084982884361</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>77</v>
       </c>
@@ -11524,7 +11524,7 @@
       </c>
       <c r="E62" s="5">
         <f t="shared" si="0"/>
-        <v>27.511177347242924</v>
+        <v>16.959761549925485</v>
       </c>
       <c r="F62" s="5">
         <v>10.551415797317437</v>
@@ -11581,7 +11581,7 @@
         <v>0.52160953800298071</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>78</v>
       </c>
@@ -11596,7 +11596,7 @@
       </c>
       <c r="E63" s="5">
         <f t="shared" si="0"/>
-        <v>64.018341755568031</v>
+        <v>38.04978476511323</v>
       </c>
       <c r="F63" s="5">
         <v>25.9685569904548</v>
@@ -11653,7 +11653,7 @@
         <v>0.77671720007486433</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>79</v>
       </c>
@@ -11668,7 +11668,7 @@
       </c>
       <c r="E64" s="5">
         <f t="shared" si="0"/>
-        <v>0.13583833148732524</v>
+        <v>4.3886230172828153E-2</v>
       </c>
       <c r="F64" s="5">
         <v>9.1952101314497089E-2</v>
@@ -11725,7 +11725,7 @@
         <v>7.7323357923554367E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>80</v>
       </c>
@@ -11740,7 +11740,7 @@
       </c>
       <c r="E65" s="5">
         <f t="shared" si="0"/>
-        <v>19.363508382748179</v>
+        <v>9.1932938014589816</v>
       </c>
       <c r="F65" s="5">
         <v>10.170214581289194</v>
@@ -11797,7 +11797,7 @@
         <v>0.28155795401220085</v>
       </c>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>81</v>
       </c>
@@ -11812,7 +11812,7 @@
       </c>
       <c r="E66" s="5">
         <f t="shared" si="0"/>
-        <v>94.991282295133928</v>
+        <v>88.968140751307658</v>
       </c>
       <c r="F66" s="5">
         <v>6.0231415438262799</v>
@@ -11869,7 +11869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>82</v>
       </c>
@@ -11883,8 +11883,8 @@
         <v>0</v>
       </c>
       <c r="E67" s="5">
-        <f t="shared" ref="E67:E94" si="4">SUM(F67:I67)</f>
-        <v>43.811240290399553</v>
+        <f t="shared" ref="E67:E94" si="4">SUM(G67:I67)</f>
+        <v>22.241965781591105</v>
       </c>
       <c r="F67" s="5">
         <v>21.569274508808448</v>
@@ -11941,7 +11941,7 @@
         <v>0.55846067929126264</v>
       </c>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>83</v>
       </c>
@@ -11956,7 +11956,7 @@
       </c>
       <c r="E68" s="5">
         <f t="shared" si="4"/>
-        <v>89.744995887030456</v>
+        <v>86.550589525637534</v>
       </c>
       <c r="F68" s="5">
         <v>3.1944063613929257</v>
@@ -12013,7 +12013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>84</v>
       </c>
@@ -12028,7 +12028,7 @@
       </c>
       <c r="E69" s="5">
         <f t="shared" si="4"/>
-        <v>93.967661691542304</v>
+        <v>91.231343283582106</v>
       </c>
       <c r="F69" s="5">
         <v>2.7363184079601992</v>
@@ -12085,7 +12085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>85</v>
       </c>
@@ -12100,7 +12100,7 @@
       </c>
       <c r="E70" s="5">
         <f t="shared" si="4"/>
-        <v>92.905675459632292</v>
+        <v>90.027977617905677</v>
       </c>
       <c r="F70" s="5">
         <v>2.877697841726619</v>
@@ -12157,7 +12157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>86</v>
       </c>
@@ -12172,7 +12172,7 @@
       </c>
       <c r="E71" s="5">
         <f t="shared" si="4"/>
-        <v>92.002176278563653</v>
+        <v>90.097932535364521</v>
       </c>
       <c r="F71" s="5">
         <v>1.9042437431991295</v>
@@ -12229,7 +12229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>87</v>
       </c>
@@ -12244,7 +12244,7 @@
       </c>
       <c r="E72" s="5">
         <f t="shared" si="4"/>
-        <v>21.680024348178961</v>
+        <v>13.640052754387746</v>
       </c>
       <c r="F72" s="5">
         <v>8.0399715937912148</v>
@@ -12301,7 +12301,7 @@
         <v>0.35000507253728314</v>
       </c>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>88</v>
       </c>
@@ -12316,7 +12316,7 @@
       </c>
       <c r="E73" s="5">
         <f t="shared" si="4"/>
-        <v>11.571458464113832</v>
+        <v>8.6210504289600323</v>
       </c>
       <c r="F73" s="5">
         <v>2.9504080351537976</v>
@@ -12373,7 +12373,7 @@
         <v>0.17786147729650553</v>
       </c>
     </row>
-    <row r="74" spans="1:22" ht="27" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:22" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>89</v>
       </c>
@@ -12388,7 +12388,7 @@
       </c>
       <c r="E74" s="5">
         <f t="shared" si="4"/>
-        <v>1.2078635126427248</v>
+        <v>0.39760703983998147</v>
       </c>
       <c r="F74" s="5">
         <v>0.81025647280274349</v>
@@ -12445,7 +12445,7 @@
         <v>2.9068408331859589E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:22" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>90</v>
       </c>
@@ -12460,7 +12460,7 @@
       </c>
       <c r="E75" s="5">
         <f t="shared" si="4"/>
-        <v>59.866570737131276</v>
+        <v>34.976126626986726</v>
       </c>
       <c r="F75" s="5">
         <v>24.89044411014455</v>
@@ -12517,7 +12517,7 @@
         <v>0.54287396167179014</v>
       </c>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:22" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>91</v>
       </c>
@@ -12532,7 +12532,7 @@
       </c>
       <c r="E76" s="5">
         <f t="shared" si="4"/>
-        <v>59.90123620455374</v>
+        <v>34.902064759884667</v>
       </c>
       <c r="F76" s="5">
         <v>24.999171444669074</v>
@@ -12589,7 +12589,7 @@
         <v>0.55016073973419943</v>
       </c>
     </row>
-    <row r="77" spans="1:22" ht="27" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:22" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>92</v>
       </c>
@@ -12604,7 +12604,7 @@
       </c>
       <c r="E77" s="5">
         <f t="shared" si="4"/>
-        <v>1.4068406446108761</v>
+        <v>0.43938479384658963</v>
       </c>
       <c r="F77" s="5">
         <v>0.96745585076428664</v>
@@ -12661,7 +12661,7 @@
         <v>2.3604708802195912E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>93</v>
       </c>
@@ -12676,7 +12676,7 @@
       </c>
       <c r="E78" s="5">
         <f t="shared" si="4"/>
-        <v>24.756537728139467</v>
+        <v>14.21274856987197</v>
       </c>
       <c r="F78" s="5">
         <v>10.543789158267503</v>
@@ -12733,7 +12733,7 @@
         <v>2.5725279215472621</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>94</v>
       </c>
@@ -12748,7 +12748,7 @@
       </c>
       <c r="E79" s="5">
         <f t="shared" si="4"/>
-        <v>6.4085045029535497</v>
+        <v>3.4398906809843015</v>
       </c>
       <c r="F79" s="5">
         <v>2.9686138219692486</v>
@@ -12805,7 +12805,7 @@
         <v>1.0759745639613079E-3</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>95</v>
       </c>
@@ -12820,7 +12820,7 @@
       </c>
       <c r="E80" s="5">
         <f t="shared" si="4"/>
-        <v>64.966685347780057</v>
+        <v>36.876517840463293</v>
       </c>
       <c r="F80" s="5">
         <v>28.090167507316771</v>
@@ -12877,7 +12877,7 @@
         <v>7.4724453577433209E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>96</v>
       </c>
@@ -12892,7 +12892,7 @@
       </c>
       <c r="E81" s="5">
         <f t="shared" si="4"/>
-        <v>57.407339246935848</v>
+        <v>33.73697964591998</v>
       </c>
       <c r="F81" s="5">
         <v>23.670359601015864</v>
@@ -12949,7 +12949,7 @@
         <v>1.4538628584047995</v>
       </c>
     </row>
-    <row r="82" spans="1:22" ht="27" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:22" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>97</v>
       </c>
@@ -12964,7 +12964,7 @@
       </c>
       <c r="E82" s="5">
         <f t="shared" si="4"/>
-        <v>8.4126226377823148</v>
+        <v>5.0075722657536046</v>
       </c>
       <c r="F82" s="5">
         <v>3.4050503720287089</v>
@@ -13021,7 +13021,7 @@
         <v>2.5103707117929808E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>98</v>
       </c>
@@ -13036,7 +13036,7 @@
       </c>
       <c r="E83" s="5">
         <f t="shared" si="4"/>
-        <v>1.820361339542536</v>
+        <v>0.76361362080477357</v>
       </c>
       <c r="F83" s="5">
         <v>1.0567477187377625</v>
@@ -13093,7 +13093,7 @@
         <v>1.7748628707139176E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>99</v>
       </c>
@@ -13108,7 +13108,7 @@
       </c>
       <c r="E84" s="5">
         <f t="shared" si="4"/>
-        <v>6.1924191361149568</v>
+        <v>3.250165039398075</v>
       </c>
       <c r="F84" s="5">
         <v>2.9422540967168813</v>
@@ -13165,7 +13165,7 @@
         <v>0.49815340154600457</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>100</v>
       </c>
@@ -13180,7 +13180,7 @@
       </c>
       <c r="E85" s="5">
         <f t="shared" si="4"/>
-        <v>2.1303994949950402</v>
+        <v>0.70376048336189012</v>
       </c>
       <c r="F85" s="5">
         <v>1.42663901163315</v>
@@ -13237,7 +13237,7 @@
         <v>0.13202272522319414</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>101</v>
       </c>
@@ -13252,7 +13252,7 @@
       </c>
       <c r="E86" s="5">
         <f t="shared" si="4"/>
-        <v>28.833856528310665</v>
+        <v>8.6617835135449379</v>
       </c>
       <c r="F86" s="5">
         <v>20.172073014765726</v>
@@ -13309,7 +13309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>102</v>
       </c>
@@ -13324,7 +13324,7 @@
       </c>
       <c r="E87" s="5">
         <f t="shared" si="4"/>
-        <v>13.456147376852222</v>
+        <v>5.4865839006808166</v>
       </c>
       <c r="F87" s="5">
         <v>7.9695634761714054</v>
@@ -13381,7 +13381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>103</v>
       </c>
@@ -13396,7 +13396,7 @@
       </c>
       <c r="E88" s="5">
         <f t="shared" si="4"/>
-        <v>17.885996409335728</v>
+        <v>6.059245960502694</v>
       </c>
       <c r="F88" s="5">
         <v>11.826750448833035</v>
@@ -13453,7 +13453,7 @@
         <v>6.7324955116696589E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>104</v>
       </c>
@@ -13468,7 +13468,7 @@
       </c>
       <c r="E89" s="5">
         <f t="shared" si="4"/>
-        <v>16.230461650308978</v>
+        <v>5.5070883315158126</v>
       </c>
       <c r="F89" s="5">
         <v>10.723373318793167</v>
@@ -13525,7 +13525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>105</v>
       </c>
@@ -13540,7 +13540,7 @@
       </c>
       <c r="E90" s="5">
         <f t="shared" si="4"/>
-        <v>20.449670882331191</v>
+        <v>7.151837881813476</v>
       </c>
       <c r="F90" s="5">
         <v>13.297833000517715</v>
@@ -13597,7 +13597,7 @@
         <v>0.19968937208786333</v>
       </c>
     </row>
-    <row r="91" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>106</v>
       </c>
@@ -13612,7 +13612,7 @@
       </c>
       <c r="E91" s="5">
         <f t="shared" si="4"/>
-        <v>10.74104912572856</v>
+        <v>3.9134054954204829</v>
       </c>
       <c r="F91" s="5">
         <v>6.8276436303080761</v>
@@ -13669,7 +13669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>107</v>
       </c>
@@ -13684,7 +13684,7 @@
       </c>
       <c r="E92" s="5">
         <f t="shared" si="4"/>
-        <v>61.242236024844722</v>
+        <v>36.024844720496894</v>
       </c>
       <c r="F92" s="5">
         <v>25.217391304347824</v>
@@ -13741,7 +13741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>108</v>
       </c>
@@ -13756,7 +13756,7 @@
       </c>
       <c r="E93" s="5">
         <f t="shared" si="4"/>
-        <v>15.885264814220072</v>
+        <v>9.9385847030517471</v>
       </c>
       <c r="F93" s="5">
         <v>5.9466801111683258</v>
@@ -13813,7 +13813,7 @@
         <v>0.13635882465869922</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>109</v>
       </c>
@@ -13828,7 +13828,7 @@
       </c>
       <c r="E94" s="5">
         <f t="shared" si="4"/>
-        <v>20.440616200099385</v>
+        <v>14.601623322842473</v>
       </c>
       <c r="F94" s="5">
         <v>5.8389928772569153</v>
@@ -13885,19 +13885,19 @@
         <v>4.1411297001822098E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.25">
       <c r="T96" s="5"/>
     </row>
-    <row r="97" spans="3:20" x14ac:dyDescent="0.3">
+    <row r="97" spans="3:20" x14ac:dyDescent="0.25">
       <c r="T97" s="5"/>
     </row>
-    <row r="98" spans="3:20" x14ac:dyDescent="0.3">
+    <row r="98" spans="3:20" x14ac:dyDescent="0.25">
       <c r="T98" s="5"/>
     </row>
-    <row r="99" spans="3:20" x14ac:dyDescent="0.3">
+    <row r="99" spans="3:20" x14ac:dyDescent="0.25">
       <c r="T99" s="5"/>
     </row>
-    <row r="100" spans="3:20" x14ac:dyDescent="0.3">
+    <row r="100" spans="3:20" x14ac:dyDescent="0.25">
       <c r="C100" s="5">
         <f>MAX(C2:C94)</f>
         <v>7.7175821505457307</v>

</xml_diff>

<commit_message>
Added function to automatically perform landcover modeling. Saved scatterplot matrix
</commit_message>
<xml_diff>
--- a/data_cache/streams_2019lulc.xlsx
+++ b/data_cache/streams_2019lulc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/530e20b7f6c3b906/Documents/KC-Streams-Analysis/data_cache/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="8_{E3052FD2-981D-4E2C-8B81-FC6F18F19128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C04F9D66-F4B5-4C77-AEE6-16CBB54E5035}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="8_{E3052FD2-981D-4E2C-8B81-FC6F18F19128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3CDEA45-EF20-479E-87A6-C23E9E9DCF06}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="13545" activeTab="1" xr2:uid="{B79C8CA6-09B2-4EB5-862A-BB01EB8BD711}"/>
+    <workbookView xWindow="28680" yWindow="-4830" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{B79C8CA6-09B2-4EB5-862A-BB01EB8BD711}"/>
   </bookViews>
   <sheets>
     <sheet name="LULC - sq m" sheetId="1" r:id="rId1"/>
@@ -7851,7 +7851,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(G11:I11)</f>
         <v>92.085822762456971</v>
       </c>
       <c r="F11" s="5">
@@ -13898,10 +13898,7 @@
       <c r="T99" s="5"/>
     </row>
     <row r="100" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C100" s="5">
-        <f>MAX(C2:C94)</f>
-        <v>7.7175821505457307</v>
-      </c>
+      <c r="C100" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>